<commit_message>
Public pages and downloads render quote chips without dealer figures
The generated site now keeps written-quote existence visible (chips, counts,
dates) while dealer-quoted figures, counters, and gap math stay off the
public pages, the xlsx/docx/pdf downloads, and the calculator seed. Data in
board.json keeps full fidelity for tooling; the redaction happens at render
and at the downloads model handoff. Also adds a python-playwright fallback
for the PDF step on environments without node playwright.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -132,13 +132,13 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -573,7 +573,7 @@
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Cheapest solid = lowest out-the-door figure (written quote where one exists, else the estimate) among live cars with a verified 1-owner / 0-accident history (or Mazda CPO) at a franchise dealer. Stretch = best-value live 2023 in the Turbo / Premium tiers, ranked by list price against KBB Seattle fair purchase price.</t>
+          <t>Cheapest solid = lowest estimated out-the-door figure among live cars with a verified 1-owner / 0-accident history (or Mazda CPO) at a franchise dealer. Stretch = best-value live 2023 in the Turbo / Premium tiers, ranked by list price against KBB Seattle fair purchase price.</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: $31,957.24 OTD, clean ($0 add-ons, $200 doc; tax + licence lumped).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>quote in preparation (Aug 11, 3:57 PM); Evan's $28,500 OTD counter sent. Oregon: email-only leverage.</t>
+          <t>quote in preparation (Aug 11, 3:57 PM); our written-number request is with the dealer. Oregon: email-only leverage.</t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>written quote Aug 11, 4:21 PM: $24,992 selling / $28,591.14 OTD, zero add-ons; accept + deposit-hold reply staged. KBB lists the dealer as “Ford of Kirkland”; same lot.</t>
+          <t>written itemized quote received Aug 11, 4:21 PM (zero add-ons, doc fee at the state cap); reply prepared. KBB lists the dealer as “Ford of Kirkland”; same lot.</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>written quote received Aug 11 (PDF, figures not yet transcribed; it lists Courtesy Guard + Forever Start add-ons); Evan countered $29,600 OTD. Oregon: email-only.</t>
+          <t>written quote received Aug 11 as a PDF; it lists Courtesy Guard + Forever Start add-ons and their removal has been requested. Oregon: email-only.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>revised written quote Aug 11, 4:43 PM: $31,000 OTD with the $995 KARR add-on struck (first sheet was $32,229.17); Evan holding at $30,200 OTD.</t>
+          <t>revised written quote received Aug 11, 4:43 PM with the KARR add-on struck; discussion ongoing.</t>
         </is>
       </c>
       <c r="Y13" s="3" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>written quote Aug 11: $31,957.24 OTD (clean sheet: $28,287 + $200 doc, $0 add-ons, tax + licence lumped at $3,470.24, not itemized); Evan countered $31,100 OTD; next ask is the itemized tax/licence.</t>
+          <t>written quote received Aug 11 (clean sheet; tax and licence lumped in one line, itemization requested); discussion ongoing.</t>
         </is>
       </c>
       <c r="Y14" s="3" t="inlineStr">
@@ -2135,7 +2135,7 @@
       <c r="W16" s="6" t="n"/>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>written $28,718.60 OTD ($25,400 selling, $0 doc, no add-ons) valid to Aug 12, 7 PM; Evan's $27,000 + inspection counter was declined.</t>
+          <t>written offer in hand, valid to Aug 12, 7 PM; Carfax shows a 6/2024 accident. Discussion paused.</t>
         </is>
       </c>
       <c r="Y16" s="3" t="inlineStr">
@@ -2321,7 +2321,7 @@
       <c r="W18" s="6" t="n"/>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>folded into the #8 thread with a $29,400 OTD counter (Aug 11); no separate quote yet. Oregon: email-only.</t>
+          <t>folded into the #8 thread; no separate quote yet. Oregon: email-only.</t>
         </is>
       </c>
       <c r="Y18" s="3" t="inlineStr">
@@ -2442,7 +2442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:T8"/>
+  <dimension ref="B1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -2584,335 +2584,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="B4" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>2021 Grand Touring AWD</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Hyundai of Kirkland / Ford of Kirkland</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Aug 11 4:21 PM PT</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>itemized written proposal (email)</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>24992</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I4" s="11" t="n">
-        <v>2699.14</v>
-      </c>
-      <c r="J4" s="10" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="K4" s="9" t="n">
-        <v>700</v>
-      </c>
-      <c r="L4" s="11" t="n"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="N4" s="11" t="n">
-        <v>28591.14</v>
-      </c>
-      <c r="O4" s="11" t="n"/>
-      <c r="P4" s="12" t="n">
-        <v>28712.736</v>
-      </c>
-      <c r="Q4" s="9" t="n">
-        <v>27700</v>
-      </c>
-      <c r="R4" s="12">
-        <f>N4-Q4</f>
-        <v/>
-      </c>
-      <c r="S4" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>selling $200 under list; zero add-ons · counter: front-runner bump via site form; superseded by the priority rule: accept any clean sheet at or under list</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>2023 2.5 S Preferred</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Royal Moore Mazda</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Aug 11 3:06 PM PT</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>pricing breakdown PDF (figures not yet transcribed)</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Courtesy Guard, Forever Start</t>
-        </is>
-      </c>
-      <c r="N5" s="11" t="n"/>
-      <c r="O5" s="11" t="n"/>
-      <c r="P5" s="12" t="n">
-        <v>30472.45</v>
-      </c>
-      <c r="Q5" s="9" t="n">
-        <v>29600</v>
-      </c>
-      <c r="R5" s="12" t="n"/>
-      <c r="S5" s="7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
-          <t>carries two dealer add-ons to strike · counter: two-car counter with #20 ($29,400)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>2022 2.5 S Premium Plus</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Titus-Will Chevrolet GMC Cadillac</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Aug 11 4:43 PM PT</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>revised written proposal (PDF)</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>27268.6</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="10" t="n"/>
-      <c r="K6" s="9" t="n">
-        <v>750</v>
-      </c>
-      <c r="L6" s="11" t="n"/>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="N6" s="11" t="n">
-        <v>31000</v>
-      </c>
-      <c r="O6" s="11" t="n">
-        <v>32229.17</v>
-      </c>
-      <c r="P6" s="12" t="n">
-        <v>30982.678</v>
-      </c>
-      <c r="Q6" s="9" t="n">
-        <v>30200</v>
-      </c>
-      <c r="R6" s="12">
-        <f>N6-Q6</f>
-        <v/>
-      </c>
-      <c r="S6" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>$995 KARR add-on struck on the revision; $750 government fees to be trued up at actuals · counter: KARR + gov-fee strikes; holding</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>2023 2.5 S Premium</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Rodland Toyota of Everett</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Aug 11 3:24 PM PT</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>'Estimated Pricing Summary' payment-estimator printout (PDF, 3 pages; not a signed buyer's order)</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>28487</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="9" t="n"/>
-      <c r="L7" s="11" t="n">
-        <v>3470.24</v>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v>31957.24</v>
-      </c>
-      <c r="O7" s="11" t="n"/>
-      <c r="P7" s="12" t="n">
-        <v>32028.848</v>
-      </c>
-      <c r="Q7" s="9" t="n">
-        <v>31100</v>
-      </c>
-      <c r="R7" s="12">
-        <f>N7-Q7</f>
-        <v/>
-      </c>
-      <c r="S7" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>tax + licence lumped, consistent with Everett 10.40% plus ~$508 of title/licence; ask for the itemized rate and licence · counter: $27,300 selling; gap $857</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>2021 Grand Touring w/ GT Premium pkg</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Auto 206 (independent)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Aug 11 1:57 PM PT</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>itemized written offer (email + PDF)</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>25400</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>2768.6</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="K8" s="9" t="n">
-        <v>550</v>
-      </c>
-      <c r="L8" s="11" t="n"/>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="N8" s="11" t="n">
-        <v>28718.6</v>
-      </c>
-      <c r="O8" s="11" t="n"/>
-      <c r="P8" s="12" t="n">
-        <v>29211.091</v>
-      </c>
-      <c r="Q8" s="9" t="n">
-        <v>27000</v>
-      </c>
-      <c r="R8" s="12">
-        <f>N8-Q8</f>
-        <v/>
-      </c>
-      <c r="S8" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="T8" s="3" t="inlineStr">
-        <is>
-          <t>cleanest fee sheet seen: no doc fee, no add-ons; disqualified by the Carfax accident unless the rule is waived · counter: contingent on a clean independent PPI; declined by the dealer</t>
-        </is>
-      </c>
-    </row>
+    <row r="4"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2971,7 +2643,7 @@
           <t>APR</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="11" t="n">
         <v>0.063</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -2979,7 +2651,7 @@
           <t>Per $1,000 financed</t>
         </is>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="12">
         <f>-PMT($C$3/12,$C$4,1000)</f>
         <v/>
       </c>
@@ -2990,10 +2662,10 @@
           <t>Term (months)</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Bankrate super-prime used-auto average, updated 7/31/26; credit-union check BECU 5.99% effective 8/1/26</t>
         </is>
@@ -3005,7 +2677,7 @@
           <t>Down payment (scenario 2)</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="15" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -3015,7 +2687,7 @@
           <t>License / title / RTA est.</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="15" t="n">
         <v>600</v>
       </c>
     </row>
@@ -3119,24 +2791,24 @@
       <c r="H9" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="I9" s="12">
+      <c r="I9" s="16">
         <f>F9*(1+G9)+H9+$C$6</f>
         <v/>
       </c>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="14">
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="12">
         <f>IF(J9&gt;0,J9,I9)</f>
         <v/>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="16">
         <f>-PMT($C$3/12,$C$4,K9)</f>
         <v/>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K9-$C$5))</f>
         <v/>
       </c>
-      <c r="N9" s="12">
+      <c r="N9" s="16">
         <f>L9*$C$4-K9</f>
         <v/>
       </c>
@@ -3174,24 +2846,24 @@
       <c r="H10" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I10" s="12">
+      <c r="I10" s="16">
         <f>F10*(1+G10)+H10+$C$6</f>
         <v/>
       </c>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="14">
+      <c r="J10" s="17" t="n"/>
+      <c r="K10" s="12">
         <f>IF(J10&gt;0,J10,I10)</f>
         <v/>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="16">
         <f>-PMT($C$3/12,$C$4,K10)</f>
         <v/>
       </c>
-      <c r="M10" s="12">
+      <c r="M10" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K10-$C$5))</f>
         <v/>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="16">
         <f>L10*$C$4-K10</f>
         <v/>
       </c>
@@ -3217,7 +2889,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>quoted</t>
+          <t>est</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
@@ -3229,104 +2901,100 @@
       <c r="H11" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="16">
         <f>F11*(1+G11)+H11+$C$6</f>
         <v/>
       </c>
-      <c r="J11" s="11" t="n">
-        <v>28591.14</v>
-      </c>
-      <c r="K11" s="14">
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="12">
         <f>IF(J11&gt;0,J11,I11)</f>
         <v/>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="16">
         <f>-PMT($C$3/12,$C$4,K11)</f>
         <v/>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K11-$C$5))</f>
         <v/>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="16">
         <f>L11*$C$4-K11</f>
         <v/>
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>Aug 11 sheet</t>
+          <t>est. at Kirkland, WA rate</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>2021 Grand Touring w/ GT Premium pkg</t>
+          <t>2021 Signature (2.5T)</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Auto 206 (independent)</t>
+          <t>Cortes Auto Center (independent)</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>quoted</t>
+          <t>est</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>25799</v>
+        <v>25999</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.109</v>
+        <v>0.091</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="12">
+        <v>200</v>
+      </c>
+      <c r="I12" s="16">
         <f>F12*(1+G12)+H12+$C$6</f>
         <v/>
       </c>
-      <c r="J12" s="11" t="n">
-        <v>28718.6</v>
-      </c>
-      <c r="K12" s="14">
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="12">
         <f>IF(J12&gt;0,J12,I12)</f>
         <v/>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="16">
         <f>-PMT($C$3/12,$C$4,K12)</f>
         <v/>
       </c>
-      <c r="M12" s="12">
+      <c r="M12" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K12-$C$5))</f>
         <v/>
       </c>
-      <c r="N12" s="12">
+      <c r="N12" s="16">
         <f>L12*$C$4-K12</f>
         <v/>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>Aug 11 sheet</t>
+          <t>est. at Burlington, WA rate</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>2021 Signature (2.5T)</t>
+          <t>2021 Grand Touring w/ GT Premium pkg</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Cortes Auto Center (independent)</t>
+          <t>Auto 206 (independent)</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3335,38 +3003,38 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>25999</v>
+        <v>25799</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>0.091</v>
+        <v>0.109</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I13" s="12">
+        <v>0</v>
+      </c>
+      <c r="I13" s="16">
         <f>F13*(1+G13)+H13+$C$6</f>
         <v/>
       </c>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="14">
+      <c r="J13" s="17" t="n"/>
+      <c r="K13" s="12">
         <f>IF(J13&gt;0,J13,I13)</f>
         <v/>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="16">
         <f>-PMT($C$3/12,$C$4,K13)</f>
         <v/>
       </c>
-      <c r="M13" s="12">
+      <c r="M13" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K13-$C$5))</f>
         <v/>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="16">
         <f>L13*$C$4-K13</f>
         <v/>
       </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>est. at Burlington, WA rate</t>
+          <t>est. at Kent, WA rate</t>
         </is>
       </c>
     </row>
@@ -3398,24 +3066,24 @@
       <c r="H14" s="9" t="n">
         <v>250</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="16">
         <f>F14*(1+G14)+H14+$C$6</f>
         <v/>
       </c>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="14">
+      <c r="J14" s="17" t="n"/>
+      <c r="K14" s="12">
         <f>IF(J14&gt;0,J14,I14)</f>
         <v/>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="16">
         <f>-PMT($C$3/12,$C$4,K14)</f>
         <v/>
       </c>
-      <c r="M14" s="12">
+      <c r="M14" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K14-$C$5))</f>
         <v/>
       </c>
-      <c r="N14" s="12">
+      <c r="N14" s="16">
         <f>L14*$C$4-K14</f>
         <v/>
       </c>
@@ -3453,24 +3121,24 @@
       <c r="H15" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="16">
         <f>F15*(1+G15)+H15+$C$6</f>
         <v/>
       </c>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="14">
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="12">
         <f>IF(J15&gt;0,J15,I15)</f>
         <v/>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="16">
         <f>-PMT($C$3/12,$C$4,K15)</f>
         <v/>
       </c>
-      <c r="M15" s="12">
+      <c r="M15" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K15-$C$5))</f>
         <v/>
       </c>
-      <c r="N15" s="12">
+      <c r="N15" s="16">
         <f>L15*$C$4-K15</f>
         <v/>
       </c>
@@ -3508,24 +3176,24 @@
       <c r="H16" s="9" t="n">
         <v>250</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="16">
         <f>F16*(1+G16)+H16+$C$6</f>
         <v/>
       </c>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="14">
+      <c r="J16" s="17" t="n"/>
+      <c r="K16" s="12">
         <f>IF(J16&gt;0,J16,I16)</f>
         <v/>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="16">
         <f>-PMT($C$3/12,$C$4,K16)</f>
         <v/>
       </c>
-      <c r="M16" s="12">
+      <c r="M16" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K16-$C$5))</f>
         <v/>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="16">
         <f>L16*$C$4-K16</f>
         <v/>
       </c>
@@ -3563,24 +3231,24 @@
       <c r="H17" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="12">
+      <c r="I17" s="16">
         <f>F17*(1+G17)+H17+$C$6</f>
         <v/>
       </c>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="14">
+      <c r="J17" s="17" t="n"/>
+      <c r="K17" s="12">
         <f>IF(J17&gt;0,J17,I17)</f>
         <v/>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="16">
         <f>-PMT($C$3/12,$C$4,K17)</f>
         <v/>
       </c>
-      <c r="M17" s="12">
+      <c r="M17" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K17-$C$5))</f>
         <v/>
       </c>
-      <c r="N17" s="12">
+      <c r="N17" s="16">
         <f>L17*$C$4-K17</f>
         <v/>
       </c>
@@ -3618,24 +3286,24 @@
       <c r="H18" s="9" t="n">
         <v>250</v>
       </c>
-      <c r="I18" s="12">
+      <c r="I18" s="16">
         <f>F18*(1+G18)+H18+$C$6</f>
         <v/>
       </c>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="14">
+      <c r="J18" s="17" t="n"/>
+      <c r="K18" s="12">
         <f>IF(J18&gt;0,J18,I18)</f>
         <v/>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="16">
         <f>-PMT($C$3/12,$C$4,K18)</f>
         <v/>
       </c>
-      <c r="M18" s="12">
+      <c r="M18" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K18-$C$5))</f>
         <v/>
       </c>
-      <c r="N18" s="12">
+      <c r="N18" s="16">
         <f>L18*$C$4-K18</f>
         <v/>
       </c>
@@ -3661,7 +3329,7 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>quoted</t>
+          <t>est</t>
         </is>
       </c>
       <c r="F19" s="9" t="n">
@@ -3673,32 +3341,30 @@
       <c r="H19" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="16">
         <f>F19*(1+G19)+H19+$C$6</f>
         <v/>
       </c>
-      <c r="J19" s="11" t="n">
-        <v>31000</v>
-      </c>
-      <c r="K19" s="14">
+      <c r="J19" s="17" t="n"/>
+      <c r="K19" s="12">
         <f>IF(J19&gt;0,J19,I19)</f>
         <v/>
       </c>
-      <c r="L19" s="12">
+      <c r="L19" s="16">
         <f>-PMT($C$3/12,$C$4,K19)</f>
         <v/>
       </c>
-      <c r="M19" s="12">
+      <c r="M19" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K19-$C$5))</f>
         <v/>
       </c>
-      <c r="N19" s="12">
+      <c r="N19" s="16">
         <f>L19*$C$4-K19</f>
         <v/>
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>Aug 11 sheet</t>
+          <t>est. at Olympia, WA rate</t>
         </is>
       </c>
     </row>
@@ -3730,24 +3396,24 @@
       <c r="H20" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="16">
         <f>F20*(1+G20)+H20+$C$6</f>
         <v/>
       </c>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="14">
+      <c r="J20" s="17" t="n"/>
+      <c r="K20" s="12">
         <f>IF(J20&gt;0,J20,I20)</f>
         <v/>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="16">
         <f>-PMT($C$3/12,$C$4,K20)</f>
         <v/>
       </c>
-      <c r="M20" s="12">
+      <c r="M20" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K20-$C$5))</f>
         <v/>
       </c>
-      <c r="N20" s="12">
+      <c r="N20" s="16">
         <f>L20*$C$4-K20</f>
         <v/>
       </c>
@@ -3785,24 +3451,24 @@
       <c r="H21" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="16">
         <f>F21*(1+G21)+H21+$C$6</f>
         <v/>
       </c>
-      <c r="J21" s="11" t="n"/>
-      <c r="K21" s="14">
+      <c r="J21" s="17" t="n"/>
+      <c r="K21" s="12">
         <f>IF(J21&gt;0,J21,I21)</f>
         <v/>
       </c>
-      <c r="L21" s="12">
+      <c r="L21" s="16">
         <f>-PMT($C$3/12,$C$4,K21)</f>
         <v/>
       </c>
-      <c r="M21" s="12">
+      <c r="M21" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K21-$C$5))</f>
         <v/>
       </c>
-      <c r="N21" s="12">
+      <c r="N21" s="16">
         <f>L21*$C$4-K21</f>
         <v/>
       </c>
@@ -3840,24 +3506,24 @@
       <c r="H22" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I22" s="12">
+      <c r="I22" s="16">
         <f>F22*(1+G22)+H22+$C$6</f>
         <v/>
       </c>
-      <c r="J22" s="11" t="n"/>
-      <c r="K22" s="14">
+      <c r="J22" s="17" t="n"/>
+      <c r="K22" s="12">
         <f>IF(J22&gt;0,J22,I22)</f>
         <v/>
       </c>
-      <c r="L22" s="12">
+      <c r="L22" s="16">
         <f>-PMT($C$3/12,$C$4,K22)</f>
         <v/>
       </c>
-      <c r="M22" s="12">
+      <c r="M22" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K22-$C$5))</f>
         <v/>
       </c>
-      <c r="N22" s="12">
+      <c r="N22" s="16">
         <f>L22*$C$4-K22</f>
         <v/>
       </c>
@@ -3938,7 +3604,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>quoted</t>
+          <t>est</t>
         </is>
       </c>
       <c r="F24" s="9" t="n">
@@ -3950,32 +3616,30 @@
       <c r="H24" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I24" s="12">
+      <c r="I24" s="16">
         <f>F24*(1+G24)+H24+$C$6</f>
         <v/>
       </c>
-      <c r="J24" s="11" t="n">
-        <v>31957.24</v>
-      </c>
-      <c r="K24" s="14">
+      <c r="J24" s="17" t="n"/>
+      <c r="K24" s="12">
         <f>IF(J24&gt;0,J24,I24)</f>
         <v/>
       </c>
-      <c r="L24" s="12">
+      <c r="L24" s="16">
         <f>-PMT($C$3/12,$C$4,K24)</f>
         <v/>
       </c>
-      <c r="M24" s="12">
+      <c r="M24" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K24-$C$5))</f>
         <v/>
       </c>
-      <c r="N24" s="12">
+      <c r="N24" s="16">
         <f>L24*$C$4-K24</f>
         <v/>
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
-          <t>Aug 11 sheet</t>
+          <t>est. at Everett, WA rate</t>
         </is>
       </c>
     </row>
@@ -4000,27 +3664,27 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="n">
-        <v>24992</v>
+          <t>est</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>25192</v>
       </c>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
-      <c r="K27" s="12" t="n">
-        <v>28591.14</v>
-      </c>
-      <c r="L27" s="12" t="n">
-        <v>556.7439727314284</v>
-      </c>
-      <c r="M27" s="12" t="n">
-        <v>459.3809482540154</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>4813.498363885701</v>
+      <c r="K27" s="16" t="n">
+        <v>28712.736</v>
+      </c>
+      <c r="L27" s="16" t="n">
+        <v>559.1117635962995</v>
+      </c>
+      <c r="M27" s="16" t="n">
+        <v>461.7487391188865</v>
+      </c>
+      <c r="N27" s="16" t="n">
+        <v>4833.969815777968</v>
       </c>
     </row>
     <row r="28">
@@ -4040,23 +3704,23 @@
           <t>est</t>
         </is>
       </c>
-      <c r="F28" s="12" t="n">
+      <c r="F28" s="16" t="n">
         <v>27999</v>
       </c>
       <c r="G28" s="7" t="n"/>
       <c r="H28" s="7" t="n"/>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="7" t="n"/>
-      <c r="K28" s="12" t="n">
+      <c r="K28" s="16" t="n">
         <v>31822.892</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="L28" s="16" t="n">
         <v>619.6746025476141</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="M28" s="16" t="n">
         <v>522.3115780702011</v>
       </c>
-      <c r="N28" s="12" t="n">
+      <c r="N28" s="16" t="n">
         <v>5357.584152856845</v>
       </c>
     </row>
@@ -4070,29 +3734,29 @@
       <c r="D29" s="25" t="n"/>
       <c r="E29" s="25" t="n"/>
       <c r="F29" s="26" t="n">
-        <v>3007</v>
+        <v>2807</v>
       </c>
       <c r="G29" s="25" t="n"/>
       <c r="H29" s="25" t="n"/>
       <c r="I29" s="25" t="n"/>
       <c r="J29" s="25" t="n"/>
       <c r="K29" s="26" t="n">
-        <v>3231.752000000004</v>
+        <v>3110.156000000003</v>
       </c>
       <c r="L29" s="26" t="n">
-        <v>62.93062981618573</v>
+        <v>60.56283895131457</v>
       </c>
       <c r="M29" s="26" t="n">
-        <v>62.93062981618573</v>
+        <v>60.56283895131463</v>
       </c>
       <c r="N29" s="26" t="n">
-        <v>544.0857889711442</v>
+        <v>523.6143370788777</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>Rule: cheapest solid = lowest out-the-door figure (written quote where one exists, else the estimate) among live cars with a verified 1-owner / 0-accident history (or Mazda CPO) at a franchise dealer; stretch = best-value live 2023 in the Turbo / Premium tiers, ranked by list price against KBB Seattle fair purchase price.</t>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Rule: cheapest solid = lowest estimated out-the-door figure among live cars with a verified 1-owner / 0-accident history (or Mazda CPO) at a franchise dealer; stretch = best-value live 2023 in the Turbo / Premium tiers, ranked by list price against KBB Seattle fair purchase price.</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4202,7 @@
       <c r="F4" s="9" t="n">
         <v>27198</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="6" t="n">
@@ -4582,7 +4246,7 @@
       <c r="F5" s="9" t="n">
         <v>24081</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="6" t="n"/>
@@ -4620,7 +4284,7 @@
       <c r="F6" s="9" t="n">
         <v>27260</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="6" t="n">
@@ -4664,7 +4328,7 @@
       <c r="F7" s="9" t="n">
         <v>28998</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="6" t="n"/>
@@ -4702,7 +4366,7 @@
       <c r="F8" s="9" t="n">
         <v>25895</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="6" t="n">
@@ -4746,7 +4410,7 @@
       <c r="F9" s="9" t="n">
         <v>25195</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
@@ -4790,7 +4454,7 @@
       <c r="F10" s="9" t="n">
         <v>27999</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n"/>
@@ -4828,7 +4492,7 @@
       <c r="F11" s="9" t="n">
         <v>27722</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n"/>
@@ -4864,7 +4528,7 @@
       <c r="F12" s="9" t="n">
         <v>27400</v>
       </c>
-      <c r="G12" s="12" t="n"/>
+      <c r="G12" s="16" t="n"/>
       <c r="H12" s="6" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="3" t="inlineStr">
@@ -4900,7 +4564,7 @@
       <c r="F13" s="9" t="n">
         <v>25950</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="16" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n"/>
@@ -5033,7 +4697,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="16">
         <f>F4-IF(E4&gt;0,E4,D4)</f>
         <v/>
       </c>
@@ -5065,7 +4729,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="16">
         <f>F5-IF(E5&gt;0,E5,D5)</f>
         <v/>
       </c>
@@ -5091,7 +4755,7 @@
       </c>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="7" t="n"/>
-      <c r="H6" s="12" t="n"/>
+      <c r="H6" s="16" t="n"/>
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="6" t="n">
         <v>0</v>
@@ -5118,7 +4782,7 @@
           <t>#6</t>
         </is>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="16">
         <f>F7-IF(E7&gt;0,E7,D7)</f>
         <v/>
       </c>
@@ -5154,7 +4818,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="16">
         <f>F8-IF(E8&gt;0,E8,D8)</f>
         <v/>
       </c>
@@ -5186,7 +4850,7 @@
           <t>#21</t>
         </is>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="16">
         <f>F9-IF(E9&gt;0,E9,D9)</f>
         <v/>
       </c>
@@ -5216,7 +4880,7 @@
           <t>CarGurus</t>
         </is>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="16">
         <f>F10-IF(E10&gt;0,E10,D10)</f>
         <v/>
       </c>
@@ -5250,7 +4914,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="16">
         <f>F11-IF(E11&gt;0,E11,D11)</f>
         <v/>
       </c>
@@ -5286,7 +4950,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="16">
         <f>F12-IF(E12&gt;0,E12,D12)</f>
         <v/>
       </c>
@@ -5318,7 +4982,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="16">
         <f>F13-IF(E13&gt;0,E13,D13)</f>
         <v/>
       </c>
@@ -5350,7 +5014,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="16">
         <f>F14-IF(E14&gt;0,E14,D14)</f>
         <v/>
       </c>
@@ -5380,7 +5044,7 @@
           <t>#10</t>
         </is>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="16">
         <f>F15-IF(E15&gt;0,E15,D15)</f>
         <v/>
       </c>
@@ -5416,7 +5080,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="16">
         <f>F16-IF(E16&gt;0,E16,D16)</f>
         <v/>
       </c>
@@ -5448,7 +5112,7 @@
           <t>CarGurus</t>
         </is>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="16">
         <f>F17-IF(E17&gt;0,E17,D17)</f>
         <v/>
       </c>
@@ -5480,7 +5144,7 @@
           <t>CarMax</t>
         </is>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="16">
         <f>F18-IF(E18&gt;0,E18,D18)</f>
         <v/>
       </c>
@@ -5512,7 +5176,7 @@
           <t>#1</t>
         </is>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="16">
         <f>F19-IF(E19&gt;0,E19,D19)</f>
         <v/>
       </c>
@@ -5522,14 +5186,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>¹ Seattle FPP = mean of per-listing kbbFppAmount from KBB search results (n=1–5 per cell).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>² No Seattle FPP for this cell; Δ shown vs national — national is systematically ~$3–5k low (default-zip, higher-mileage assumption), so treat these as “at market,” not overpriced.</t>
         </is>

</xml_diff>

<commit_message>
Board: Lee Johnson inquiry emails bounced; status reflects undelivered requests
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O20"/>
+  <dimension ref="B1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -604,61 +604,68 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -1347,7 +1354,7 @@
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>two-car OTD request (#7 + #12) emailed Aug 11, 3:50 PM; no reply yet.</t>
+          <t>two-car OTD request emailed Aug 11 — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
         </is>
       </c>
       <c r="Y8" s="3" t="inlineStr">
@@ -1741,7 +1748,7 @@
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>in the Lee Johnson two-car OTD request emailed Aug 11, 3:50 PM; no reply yet.</t>
+          <t>in the Lee Johnson two-car OTD request (Aug 11) — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
         </is>
       </c>
       <c r="Y12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Board: Puyallup written quotes in hand for two cars; third requested
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O21"/>
+  <dimension ref="B1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>16 cars in play (15 live + benchmark), 5 sold since publication, 5 written quotes in hand.</t>
+          <t>16 cars in play (15 live + benchmark), 5 sold since publication, 7 written quotes in hand.</t>
         </is>
       </c>
     </row>
@@ -604,68 +604,75 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -948,7 +955,7 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>awaiting written OTD; form lead Aug 11 plus a phone promise, nothing received.</t>
+          <t>written itemized quote in hand (sheet dated Aug 11, surfaced Aug 12 after a phone call; the sender's group domain had gone to spam); zero add-ons.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
@@ -1252,7 +1259,7 @@
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>awaiting written OTD; same Puyallup lead as #1 (Aug 11), phone promise only.</t>
+          <t>written itemized quote in hand (sheet dated Aug 11, surfaced Aug 12); zero add-ons.</t>
         </is>
       </c>
       <c r="Y7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Board: Kirkland sends an updated written proposal; terms confirmations noted
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O22"/>
+  <dimension ref="B1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,7 @@
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Published Aug 7, 2026; refreshed Aug 12, 2026. Generated from data/board.json by tools/build_site.py — same rows as the web page.</t>
+          <t>Published Aug 7, 2026; refreshed Aug 13, 2026. Generated from data/board.json by tools/build_site.py — same rows as the web page.</t>
         </is>
       </c>
     </row>
@@ -604,75 +604,82 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
+          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -723,7 +730,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Board — cars in play as of Aug 12, 2026 (sold cars on their own tab)</t>
+          <t>Board — cars in play as of Aug 13, 2026 (sold cars on their own tab)</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -1159,7 +1166,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>written itemized quote received Aug 11, 4:21 PM (zero add-ons, doc fee at the state cap); reply prepared. KBB lists the dealer as “Ford of Kirkland”; same lot.</t>
+          <t>updated written proposal received Thu Aug 13 midday; license billed at actuals with any overage refunded and two keys confirmed in writing; window sticker being pulled to confirm the GT Premium package.</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
@@ -4140,7 +4147,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Watchlist: screened, not on the board (re-checked Aug 12, 2026)</t>
+          <t>Watchlist: screened, not on the board (re-checked Aug 13, 2026)</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -5001,7 +5008,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>KBB fair purchase price vs. lowest clean live listing (Aug 12, 2026)</t>
+          <t>KBB fair purchase price vs. lowest clean live listing (Aug 13, 2026)</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>

</xml_diff>

<commit_message>
Board: Puyallup CPO breakdown received; Royal Moore manager follow-up noted
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O23"/>
+  <dimension ref="B1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -604,82 +604,96 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
+          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
+          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -1470,7 +1484,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>written quote received Aug 11 as a PDF; it lists Courtesy Guard + Forever Start add-ons and their removal has been requested. Oregon: email-only.</t>
+          <t>a sales manager followed up Thu afternoon; reply prepared.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
@@ -1572,7 +1586,7 @@
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>folded into the Puyallup #1/#6 inquiry; no written numbers yet.</t>
+          <t>CPO pricing breakdown received Thu Aug 13 early afternoon; itemized worksheet attached in the dealer's email.</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Board: reply stamps for Kirkland and Royal Moore
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -1180,7 +1180,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>updated written proposal received Thu Aug 13 midday; license billed at actuals with any overage refunded and two keys confirmed in writing; window sticker being pulled to confirm the GT Premium package.</t>
+          <t>updated written proposal received Thu Aug 13 midday; license billed at actuals with any overage refunded and two keys confirmed in writing; window sticker being pulled to confirm the GT Premium package; replied Thu afternoon.</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>a sales manager followed up Thu afternoon; reply prepared.</t>
+          <t>a sales manager followed up Thu afternoon; replied Thu afternoon.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Board: Royal Moore reports one Preferred sold; the other requoted with add-ons removed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O25"/>
+  <dimension ref="B1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>16 cars in play (15 live + benchmark), 5 sold since publication, 7 written quotes in hand.</t>
+          <t>15 cars in play (14 live + benchmark), 6 sold since publication, 6 written quotes in hand.</t>
         </is>
       </c>
     </row>
@@ -604,96 +604,103 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
+          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
+          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
+          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
+          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -711,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Y19"/>
+  <dimension ref="B1:Y18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -1393,7 +1400,7 @@
     </row>
     <row r="9">
       <c r="B9" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
@@ -1405,7 +1412,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred</t>
+          <t>2.5 S Carbon Edition</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1414,37 +1421,37 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>16615</v>
+        <v>33006</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>26900</v>
+        <v>27699</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>26900</v>
+        <v>27499</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Royal Moore Mazda</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Hillsboro, OR</t>
+          <t>Puyallup, WA</t>
         </is>
       </c>
       <c r="M9" s="10" t="n">
-        <v>0.1105</v>
+        <v>0.108</v>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>Good · $469 below</t>
+          <t>Good · $518 below</t>
         </is>
       </c>
       <c r="O9" s="9" t="n">
-        <v>27590</v>
+        <v>28090</v>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
@@ -1453,11 +1460,11 @@
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R9" s="6" t="n">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
@@ -1466,36 +1473,36 @@
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/454567468</t>
+          <t>https://www.cargurus.com/Cars/listing/450917825</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCM6P0274841</t>
+          <t>JM3KFBCMXP0288130</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>661788A</t>
+          <t>M260362A</t>
         </is>
       </c>
       <c r="W9" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>a sales manager followed up Thu afternoon; replied Thu afternoon.</t>
+          <t>CPO pricing breakdown received Thu Aug 13 early afternoon; itemized worksheet attached in the dealer's email.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t>Leatherette, heated fronts, power driver seat, moonroof.</t>
+          <t>Red leather, heated fronts, Mazda CPO warranty.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
@@ -1507,7 +1514,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Carbon Edition</t>
+          <t>2.5 S Preferred</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1516,88 +1523,86 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>33006</v>
+        <v>44989</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>27699</v>
+        <v>24095</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>27499</v>
+        <v>23995</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Puyallup Mazda</t>
+          <t>Columbia Sales &amp; Service</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>Puyallup, WA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="M10" s="10" t="n">
-        <v>0.108</v>
+        <v>0.1105</v>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>Good · $518 below</t>
-        </is>
-      </c>
-      <c r="O10" s="9" t="n">
-        <v>28090</v>
-      </c>
+          <t>Great · Cars.com rating</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="n"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 0 accidents</t>
+          <t>2 owners · 0 accidents</t>
         </is>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R10" s="6" t="n">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="S10" s="7" t="inlineStr">
         <is>
-          <t>CarGurus</t>
+          <t>Cars.com</t>
         </is>
       </c>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/450917825</t>
+          <t>https://www.cars.com/vehicledetail/d4fd9d01-99f9-4673-87c0-1a173ef9551f/</t>
         </is>
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCMXP0288130</t>
+          <t>JM3KFBCM9P0119426</t>
         </is>
       </c>
       <c r="V10" s="7" t="inlineStr">
         <is>
-          <t>M260362A</t>
+          <t>2468</t>
         </is>
       </c>
       <c r="W10" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>CPO pricing breakdown received Thu Aug 13 early afternoon; itemized worksheet attached in the dealer's email.</t>
+          <t>emailed Aug 11, no reply. Oregon: email-only.</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
-          <t>Red leather, heated fronts, Mazda CPO warranty.</t>
+          <t>Leatherette, heated fronts, moonroof.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
@@ -1609,7 +1614,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred</t>
+          <t>2.5 S Preferred · Mazda CPO</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1618,49 +1623,43 @@
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>44989</v>
+        <v>36400</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>24095</v>
+        <v>26348</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>23995</v>
+        <v>26348</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Columbia Sales &amp; Service</t>
+          <t>Lee Johnson Mazda of Seattle</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="M11" s="10" t="n">
         <v>0.1105</v>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>Great · Cars.com rating</t>
-        </is>
-      </c>
+      <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="9" t="n"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2 owners · 0 accidents</t>
+          <t>0 accidents</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>29</v>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="n"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
           <t>Cars.com</t>
@@ -1668,36 +1667,32 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/d4fd9d01-99f9-4673-87c0-1a173ef9551f/</t>
+          <t>https://www.cars.com/vehicledetail/d7b0a899-fdc8-4776-9379-64684c757f41/</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCM9P0119426</t>
-        </is>
-      </c>
-      <c r="V11" s="7" t="inlineStr">
-        <is>
-          <t>2468</t>
-        </is>
-      </c>
+          <t>JM3KFBCM7P0256994</t>
+        </is>
+      </c>
+      <c r="V11" s="7" t="n"/>
       <c r="W11" s="6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>emailed Aug 11, no reply. Oregon: email-only.</t>
+          <t>in the Lee Johnson two-car OTD request (Aug 11) — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
         </is>
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>Leatherette, heated fronts, moonroof.</t>
+          <t>Leather-trimmed Preferred content (heated fronts, moonroof) with the Mazda CPO warranty.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
@@ -1705,11 +1700,11 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred · Mazda CPO</t>
+          <t>2.5 S Premium Plus</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1718,76 +1713,88 @@
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>36400</v>
+        <v>43640</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>26348</v>
+        <v>27389</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>26348</v>
+        <v>27389</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Lee Johnson Mazda of Seattle</t>
+          <t>Titus-Will Chevrolet GMC Cadillac</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Olympia, WA</t>
         </is>
       </c>
       <c r="M12" s="10" t="n">
-        <v>0.1105</v>
-      </c>
-      <c r="N12" s="7" t="inlineStr"/>
-      <c r="O12" s="9" t="n"/>
+        <v>0.102</v>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>Good · $389 over FPP</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>27000</v>
+      </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>0 accidents</t>
+          <t>1 owner · 0 accidents</t>
         </is>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="R12" s="6" t="n"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>45</v>
+      </c>
       <c r="S12" s="7" t="inlineStr">
         <is>
-          <t>Cars.com</t>
+          <t>KBB</t>
         </is>
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/d7b0a899-fdc8-4776-9379-64684c757f41/</t>
+          <t>https://www.kbb.com/cars-for-sale/vehicle/784195725</t>
         </is>
       </c>
       <c r="U12" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCM7P0256994</t>
-        </is>
-      </c>
-      <c r="V12" s="7" t="n"/>
+          <t>JM3KFBEM1N0590576</t>
+        </is>
+      </c>
+      <c r="V12" s="7" t="inlineStr">
+        <is>
+          <t>P11101</t>
+        </is>
+      </c>
       <c r="W12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>in the Lee Johnson two-car OTD request (Aug 11) — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
+          <t>dealer asking to schedule a Saturday time (Aug 12 evening); paperwork requested first.</t>
         </is>
       </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>Leather-trimmed Preferred content (heated fronts, moonroof) with the Mazda CPO warranty.</t>
+          <t>Ventilated seats, HUD, heated rears; CarBravo (GM) certified, not Mazda CPO.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
@@ -1795,11 +1802,11 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Premium Plus</t>
+          <t>2.5 S Premium</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1808,37 +1815,37 @@
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>43640</v>
+        <v>17505</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>27389</v>
+        <v>28487</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>27389</v>
+        <v>28287</v>
       </c>
       <c r="J13" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Titus-Will Chevrolet GMC Cadillac</t>
+          <t>Rodland Toyota of Everett</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>Olympia, WA</t>
+          <t>Everett, WA</t>
         </is>
       </c>
       <c r="M13" s="10" t="n">
-        <v>0.102</v>
+        <v>0.104</v>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>Good · $389 over FPP</t>
+          <t>Good · $873 below</t>
         </is>
       </c>
       <c r="O13" s="9" t="n">
-        <v>27000</v>
+        <v>27750</v>
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
@@ -1851,49 +1858,49 @@
         </is>
       </c>
       <c r="R13" s="6" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>KBB</t>
+          <t>CarGurus</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>https://www.kbb.com/cars-for-sale/vehicle/784195725</t>
+          <t>https://www.cargurus.com/Cars/listing/453332129</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBEM1N0590576</t>
+          <t>JM3KFBDM7P0281828</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>P11101</t>
+          <t>68987A</t>
         </is>
       </c>
       <c r="W13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>dealer asking to schedule a Saturday time (Aug 12 evening); paperwork requested first.</t>
+          <t>dealer declined to negotiate by email (Aug 12 evening); no visit planned.</t>
         </is>
       </c>
       <c r="Y13" s="3" t="inlineStr">
         <is>
-          <t>Ventilated seats, HUD, heated rears; CarBravo (GM) certified, not Mazda CPO.</t>
+          <t>Lowest-mile comfort car in the set: Soul Red, leather, Bose, heated wheel (no ventilation).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
@@ -1901,7 +1908,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Premium</t>
+          <t>2.5 S Premium · no-haggle</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -1910,38 +1917,36 @@
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>17505</v>
+        <v>31166</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>28487</v>
+        <v>27998</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>28287</v>
+        <v>27998</v>
       </c>
       <c r="J14" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Rodland Toyota of Everett</t>
+          <t>CarMax Renton</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>Everett, WA</t>
+          <t>Renton, WA</t>
         </is>
       </c>
       <c r="M14" s="10" t="n">
-        <v>0.104</v>
+        <v>0.11</v>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>Good · $873 below</t>
-        </is>
-      </c>
-      <c r="O14" s="9" t="n">
-        <v>27750</v>
-      </c>
+          <t>Fair · $222 below</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="n"/>
       <c r="P14" s="7" t="inlineStr">
         <is>
           <t>1 owner · 0 accidents</t>
@@ -1953,57 +1958,57 @@
         </is>
       </c>
       <c r="R14" s="6" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="S14" s="7" t="inlineStr">
         <is>
-          <t>CarGurus</t>
+          <t>CarMax</t>
         </is>
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/453332129</t>
+          <t>https://www.cargurus.com/Cars/listing/455754266</t>
         </is>
       </c>
       <c r="U14" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM7P0281828</t>
+          <t>JM3KFBDM0P0215315</t>
         </is>
       </c>
       <c r="V14" s="7" t="inlineStr">
         <is>
-          <t>68987A</t>
+          <t>70134808</t>
         </is>
       </c>
       <c r="W14" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>dealer declined to negotiate by email (Aug 12 evening); no visit planned.</t>
+          <t>reference car; nothing to request.</t>
         </is>
       </c>
       <c r="Y14" s="3" t="inlineStr">
         <is>
-          <t>Lowest-mile comfort car in the set: Soul Red, leather, Bose, heated wheel (no ventilation).</t>
+          <t>In-state no-haggle benchmark, no transfer fee.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>benchmark</t>
+          <t>live</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Premium · no-haggle</t>
+          <t>Grand Touring w/ GT Premium pkg</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -2012,39 +2017,41 @@
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>31166</v>
+        <v>30066</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>27998</v>
+        <v>25799</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>27998</v>
+        <v>25799</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>CarMax Renton</t>
+          <t>Auto 206 (independent)</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>Renton, WA</t>
+          <t>Kent, WA</t>
         </is>
       </c>
       <c r="M15" s="10" t="n">
-        <v>0.11</v>
+        <v>0.109</v>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>Fair · $222 below</t>
-        </is>
-      </c>
-      <c r="O15" s="9" t="n"/>
+          <t>$3,281 &lt; FPP</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="n">
+        <v>29080</v>
+      </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 0 accidents</t>
+          <t>1 owner · 1 accident</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
@@ -2053,45 +2060,43 @@
         </is>
       </c>
       <c r="R15" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>CarMax</t>
+          <t>Autotrader</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/455754266</t>
+          <t>https://www.autotrader.com/cars-for-sale/vehicle/787629893</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM0P0215315</t>
+          <t>JM3KFBDM0M0305902</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>70134808</t>
-        </is>
-      </c>
-      <c r="W15" s="6" t="n">
-        <v>6</v>
-      </c>
+          <t>13014</t>
+        </is>
+      </c>
+      <c r="W15" s="6" t="n"/>
       <c r="X15" s="3" t="inlineStr">
         <is>
-          <t>reference car; nothing to request.</t>
+          <t>written offer in hand, valid to Aug 12, 7 PM; Carfax shows a 6/2024 accident. Discussion paused.</t>
         </is>
       </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
-          <t>In-state no-haggle benchmark, no transfer fee.</t>
+          <t>Ventilated seats at GT money (GT Premium package), Deep Crystal Blue.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
@@ -2103,50 +2108,50 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Grand Touring w/ GT Premium pkg</t>
+          <t>Signature (2.5T, ventilated)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5 Turbo</t>
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>30066</v>
+        <v>40451</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>25799</v>
+        <v>26712</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>25799</v>
+        <v>26712</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Auto 206 (independent)</t>
+          <t>Tonkin Gresham Honda</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>Kent, WA</t>
+          <t>Troutdale, OR</t>
         </is>
       </c>
       <c r="M16" s="10" t="n">
-        <v>0.109</v>
+        <v>0.1105</v>
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>$3,281 &lt; FPP</t>
+          <t>Good · $700 below</t>
         </is>
       </c>
       <c r="O16" s="9" t="n">
-        <v>29080</v>
+        <v>24480</v>
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 1 accident</t>
+          <t>2 owners · 0 accidents</t>
         </is>
       </c>
       <c r="Q16" s="7" t="inlineStr">
@@ -2155,43 +2160,43 @@
         </is>
       </c>
       <c r="R16" s="6" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="S16" s="7" t="inlineStr">
         <is>
-          <t>Autotrader</t>
+          <t>Cars.com</t>
         </is>
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>https://www.autotrader.com/cars-for-sale/vehicle/787629893</t>
+          <t>https://www.cars.com/vehicledetail/671f18d1-7917-4929-b9c7-3f175ba4013f/</t>
         </is>
       </c>
       <c r="U16" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM0M0305902</t>
+          <t>JM3KFBEY2M0349546</t>
         </is>
       </c>
       <c r="V16" s="7" t="inlineStr">
         <is>
-          <t>13014</t>
+          <t>G6186020B</t>
         </is>
       </c>
       <c r="W16" s="6" t="n"/>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>written offer in hand, valid to Aug 12, 7 PM; Carfax shows a 6/2024 accident. Discussion paused.</t>
+          <t>not contacted; Oregon fallback, email-only.</t>
         </is>
       </c>
       <c r="Y16" s="3" t="inlineStr">
         <is>
-          <t>Ventilated seats at GT money (GT Premium package), Deep Crystal Blue.</t>
+          <t>Top 2021 trim (Nappa, vents, 360 camera).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -2199,54 +2204,48 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Signature (2.5T, ventilated)</t>
+          <t>2.5 S Preferred</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>2.5 Turbo</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>40451</v>
+        <v>16969</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>26712</v>
+        <v>26500</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>26712</v>
+        <v>26500</v>
       </c>
       <c r="J17" s="9" t="n">
         <v>250</v>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>Tonkin Gresham Honda</t>
+          <t>Royal Moore Mazda</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Troutdale, OR</t>
+          <t>Hillsboro, OR</t>
         </is>
       </c>
       <c r="M17" s="10" t="n">
         <v>0.1105</v>
       </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>Good · $700 below</t>
-        </is>
-      </c>
-      <c r="O17" s="9" t="n">
-        <v>24480</v>
-      </c>
+      <c r="N17" s="7" t="inlineStr"/>
+      <c r="O17" s="9" t="n"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>2 owners · 0 accidents</t>
+          <t>0 accidents</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
@@ -2264,34 +2263,26 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/671f18d1-7917-4929-b9c7-3f175ba4013f/</t>
-        </is>
-      </c>
-      <c r="U17" s="7" t="inlineStr">
-        <is>
-          <t>JM3KFBEY2M0349546</t>
-        </is>
-      </c>
-      <c r="V17" s="7" t="inlineStr">
-        <is>
-          <t>G6186020B</t>
-        </is>
-      </c>
+          <t>https://www.cars.com/vehicledetail/84b6552a-4a94-4c5b-96bf-0b3b37cc55a9/</t>
+        </is>
+      </c>
+      <c r="U17" s="7" t="n"/>
+      <c r="V17" s="7" t="n"/>
       <c r="W17" s="6" t="n"/>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t>not contacted; Oregon fallback, email-only.</t>
+          <t>dealer requoted their remaining 2023 Preferred (stock p12315) Thu Aug 13 with the dealer-added items removed.</t>
         </is>
       </c>
       <c r="Y17" s="3" t="inlineStr">
         <is>
-          <t>Top 2021 trim (Nappa, vents, 360 camera).</t>
+          <t>The Royal Moore group's second low-mile Preferred (Toyota store, same auto center as #8).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
@@ -2299,48 +2290,54 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred</t>
+          <t>Signature (2.5T)</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5 Turbo</t>
         </is>
       </c>
       <c r="G18" s="6" t="n">
-        <v>16969</v>
+        <v>35589</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>26500</v>
+        <v>25999</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>26500</v>
+        <v>25999</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>Royal Moore Mazda</t>
+          <t>Cortes Auto Center (independent)</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
-          <t>Hillsboro, OR</t>
+          <t>Burlington, WA</t>
         </is>
       </c>
       <c r="M18" s="10" t="n">
-        <v>0.1105</v>
-      </c>
-      <c r="N18" s="7" t="inlineStr"/>
-      <c r="O18" s="9" t="n"/>
+        <v>0.091</v>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Good · $789 over FPP</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="n">
+        <v>25410</v>
+      </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>0 accidents</t>
+          <t>1 owner · 0 accidents</t>
         </is>
       </c>
       <c r="Q18" s="7" t="inlineStr">
@@ -2349,127 +2346,35 @@
         </is>
       </c>
       <c r="R18" s="6" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="S18" s="7" t="inlineStr">
         <is>
-          <t>Cars.com</t>
+          <t>KBB</t>
         </is>
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/84b6552a-4a94-4c5b-96bf-0b3b37cc55a9/</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
+          <t>https://www.kbb.com/cars-for-sale/vehicle/787933636</t>
+        </is>
+      </c>
+      <c r="U18" s="7" t="inlineStr">
+        <is>
+          <t>JM3KFBEY0M0417715</t>
+        </is>
+      </c>
+      <c r="V18" s="7" t="inlineStr">
+        <is>
+          <t>B1851</t>
+        </is>
+      </c>
       <c r="W18" s="6" t="n"/>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>folded into the #8 thread; no separate quote yet. Oregon: email-only.</t>
+          <t>not contacted (found Aug 12).</t>
         </is>
       </c>
       <c r="Y18" s="3" t="inlineStr">
-        <is>
-          <t>The Royal Moore group's second low-mile Preferred (Toyota store, same auto center as #8).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Signature (2.5T)</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>2.5 Turbo</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>35589</v>
-      </c>
-      <c r="H19" s="9" t="n">
-        <v>25999</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>25999</v>
-      </c>
-      <c r="J19" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>Cortes Auto Center (independent)</t>
-        </is>
-      </c>
-      <c r="L19" s="7" t="inlineStr">
-        <is>
-          <t>Burlington, WA</t>
-        </is>
-      </c>
-      <c r="M19" s="10" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>Good · $789 over FPP</t>
-        </is>
-      </c>
-      <c r="O19" s="9" t="n">
-        <v>25410</v>
-      </c>
-      <c r="P19" s="7" t="inlineStr">
-        <is>
-          <t>1 owner · 0 accidents</t>
-        </is>
-      </c>
-      <c r="Q19" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="7" t="inlineStr">
-        <is>
-          <t>KBB</t>
-        </is>
-      </c>
-      <c r="T19" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kbb.com/cars-for-sale/vehicle/787933636</t>
-        </is>
-      </c>
-      <c r="U19" s="7" t="inlineStr">
-        <is>
-          <t>JM3KFBEY0M0417715</t>
-        </is>
-      </c>
-      <c r="V19" s="7" t="inlineStr">
-        <is>
-          <t>B1851</t>
-        </is>
-      </c>
-      <c r="W19" s="6" t="n"/>
-      <c r="X19" s="3" t="inlineStr">
-        <is>
-          <t>not contacted (found Aug 12).</t>
-        </is>
-      </c>
-      <c r="Y19" s="3" t="inlineStr">
         <is>
           <t>WA car, top 2021 trim (Nappa leather, ventilated fronts, 360 camera, turbo), Snowflake White / Caturra Brown.</t>
         </is>
@@ -2642,7 +2547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O31"/>
+  <dimension ref="B1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -3250,16 +3155,16 @@
     </row>
     <row r="17">
       <c r="B17" s="6" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>2023 2.5 S Preferred</t>
+          <t>2021 Signature (2.5T, ventilated)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Royal Moore Mazda</t>
+          <t>Tonkin Gresham Honda</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -3268,13 +3173,13 @@
         </is>
       </c>
       <c r="F17" s="9" t="n">
-        <v>26900</v>
+        <v>26712</v>
       </c>
       <c r="G17" s="10" t="n">
         <v>0.1105</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="I17" s="16">
         <f>F17*(1+G17)+H17+$C$6</f>
@@ -3299,22 +3204,22 @@
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
-          <t>est. at Hillsboro, OR rate</t>
+          <t>est. at Troutdale, OR rate</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>2021 Signature (2.5T, ventilated)</t>
+          <t>2022 2.5 S Premium Plus</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Tonkin Gresham Honda</t>
+          <t>Titus-Will Chevrolet GMC Cadillac</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -3323,13 +3228,13 @@
         </is>
       </c>
       <c r="F18" s="9" t="n">
-        <v>26712</v>
+        <v>27389</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.1105</v>
+        <v>0.102</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="I18" s="16">
         <f>F18*(1+G18)+H18+$C$6</f>
@@ -3354,22 +3259,22 @@
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>est. at Troutdale, OR rate</t>
+          <t>est. at Olympia, WA rate</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="6" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>2022 2.5 S Premium Plus</t>
+          <t>2023 2.5 S Carbon Edition</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Titus-Will Chevrolet GMC Cadillac</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -3378,10 +3283,10 @@
         </is>
       </c>
       <c r="F19" s="9" t="n">
-        <v>27389</v>
+        <v>27499</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>0.102</v>
+        <v>0.108</v>
       </c>
       <c r="H19" s="9" t="n">
         <v>200</v>
@@ -3409,22 +3314,22 @@
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>est. at Olympia, WA rate</t>
+          <t>est. at Puyallup, WA rate</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>2023 2.5 S Carbon Edition</t>
+          <t>2022 2.5 S Carbon Edition</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Puyallup Mazda</t>
+          <t>Lee Johnson Mazda of Seattle</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -3433,10 +3338,10 @@
         </is>
       </c>
       <c r="F20" s="9" t="n">
-        <v>27499</v>
+        <v>27512</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.108</v>
+        <v>0.1105</v>
       </c>
       <c r="H20" s="9" t="n">
         <v>200</v>
@@ -3464,22 +3369,22 @@
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>est. at Puyallup, WA rate</t>
+          <t>est. at Seattle, WA rate</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>2022 2.5 S Carbon Edition</t>
+          <t>2023 2.5 Turbo AWD</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Lee Johnson Mazda of Seattle</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -3488,10 +3393,10 @@
         </is>
       </c>
       <c r="F21" s="9" t="n">
-        <v>27512</v>
+        <v>27999</v>
       </c>
       <c r="G21" s="10" t="n">
-        <v>0.1105</v>
+        <v>0.108</v>
       </c>
       <c r="H21" s="9" t="n">
         <v>200</v>
@@ -3519,192 +3424,174 @@
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
-          <t>est. at Seattle, WA rate</t>
+          <t>est. at Puyallup, WA rate</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>2023 2.5 Turbo AWD</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Puyallup Mazda</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="B22" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>2023 2.5 S Premium · no-haggle (benchmark)</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>CarMax Renton</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n">
-        <v>27999</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="H22" s="9" t="n">
+      <c r="F22" s="20" t="n">
+        <v>27998</v>
+      </c>
+      <c r="G22" s="21" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H22" s="20" t="n">
         <v>200</v>
       </c>
-      <c r="I22" s="16">
+      <c r="I22" s="22">
         <f>F22*(1+G22)+H22+$C$6</f>
         <v/>
       </c>
-      <c r="J22" s="17" t="n"/>
-      <c r="K22" s="12">
+      <c r="J22" s="23" t="n"/>
+      <c r="K22" s="24">
         <f>IF(J22&gt;0,J22,I22)</f>
         <v/>
       </c>
-      <c r="L22" s="16">
+      <c r="L22" s="22">
         <f>-PMT($C$3/12,$C$4,K22)</f>
         <v/>
       </c>
-      <c r="M22" s="16">
+      <c r="M22" s="22">
         <f>-PMT($C$3/12,$C$4,MAX(0,K22-$C$5))</f>
         <v/>
       </c>
-      <c r="N22" s="16">
+      <c r="N22" s="22">
         <f>L22*$C$4-K22</f>
         <v/>
       </c>
-      <c r="O22" s="7" t="inlineStr">
-        <is>
-          <t>est. at Puyallup, WA rate</t>
+      <c r="O22" s="19" t="inlineStr">
+        <is>
+          <t>est. at Renton, WA rate</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C23" s="19" t="inlineStr">
-        <is>
-          <t>2023 2.5 S Premium · no-haggle (benchmark)</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>CarMax Renton</t>
-        </is>
-      </c>
-      <c r="E23" s="19" t="inlineStr">
+      <c r="B23" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>2023 2.5 S Premium</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Rodland Toyota of Everett</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
-      <c r="F23" s="20" t="n">
-        <v>27998</v>
-      </c>
-      <c r="G23" s="21" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="H23" s="20" t="n">
+      <c r="F23" s="9" t="n">
+        <v>28287</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="H23" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I23" s="22">
+      <c r="I23" s="16">
         <f>F23*(1+G23)+H23+$C$6</f>
         <v/>
       </c>
-      <c r="J23" s="23" t="n"/>
-      <c r="K23" s="24">
+      <c r="J23" s="17" t="n"/>
+      <c r="K23" s="12">
         <f>IF(J23&gt;0,J23,I23)</f>
         <v/>
       </c>
-      <c r="L23" s="22">
+      <c r="L23" s="16">
         <f>-PMT($C$3/12,$C$4,K23)</f>
         <v/>
       </c>
-      <c r="M23" s="22">
+      <c r="M23" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K23-$C$5))</f>
         <v/>
       </c>
-      <c r="N23" s="22">
+      <c r="N23" s="16">
         <f>L23*$C$4-K23</f>
         <v/>
       </c>
-      <c r="O23" s="19" t="inlineStr">
-        <is>
-          <t>est. at Renton, WA rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>2023 2.5 S Premium</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Rodland Toyota of Everett</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>est. at Everett, WA rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Cheapest solid vs. stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Cheapest solid</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>#5 2021 Grand Touring AWD · Hyundai of Kirkland</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
-      <c r="F24" s="9" t="n">
-        <v>28287</v>
-      </c>
-      <c r="G24" s="10" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I24" s="16">
-        <f>F24*(1+G24)+H24+$C$6</f>
-        <v/>
-      </c>
-      <c r="J24" s="17" t="n"/>
-      <c r="K24" s="12">
-        <f>IF(J24&gt;0,J24,I24)</f>
-        <v/>
-      </c>
-      <c r="L24" s="16">
-        <f>-PMT($C$3/12,$C$4,K24)</f>
-        <v/>
-      </c>
-      <c r="M24" s="16">
-        <f>-PMT($C$3/12,$C$4,MAX(0,K24-$C$5))</f>
-        <v/>
-      </c>
-      <c r="N24" s="16">
-        <f>L24*$C$4-K24</f>
-        <v/>
-      </c>
-      <c r="O24" s="7" t="inlineStr">
-        <is>
-          <t>est. at Everett, WA rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Cheapest solid vs. stretch</t>
-        </is>
+      <c r="F26" s="16" t="n">
+        <v>25192</v>
+      </c>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="7" t="n"/>
+      <c r="K26" s="16" t="n">
+        <v>28712.736</v>
+      </c>
+      <c r="L26" s="16" t="n">
+        <v>559.1117635962995</v>
+      </c>
+      <c r="M26" s="16" t="n">
+        <v>461.7487391188865</v>
+      </c>
+      <c r="N26" s="16" t="n">
+        <v>4833.969815777968</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Cheapest solid</t>
+          <t>Stretch</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>#5 2021 Grand Touring AWD · Hyundai of Kirkland</t>
+          <t>#1 2023 2.5 Turbo AWD · Puyallup Mazda</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -3713,93 +3600,56 @@
         </is>
       </c>
       <c r="F27" s="16" t="n">
-        <v>25192</v>
+        <v>27999</v>
       </c>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="16" t="n">
-        <v>28712.736</v>
+        <v>31822.892</v>
       </c>
       <c r="L27" s="16" t="n">
-        <v>559.1117635962995</v>
+        <v>619.6746025476141</v>
       </c>
       <c r="M27" s="16" t="n">
-        <v>461.7487391188865</v>
+        <v>522.3115780702011</v>
       </c>
       <c r="N27" s="16" t="n">
-        <v>4833.969815777968</v>
+        <v>5357.584152856845</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>#1 2023 2.5 Turbo AWD · Puyallup Mazda</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>est</t>
-        </is>
-      </c>
-      <c r="F28" s="16" t="n">
-        <v>27999</v>
-      </c>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="n"/>
-      <c r="K28" s="16" t="n">
-        <v>31822.892</v>
-      </c>
-      <c r="L28" s="16" t="n">
-        <v>619.6746025476141</v>
-      </c>
-      <c r="M28" s="16" t="n">
-        <v>522.3115780702011</v>
-      </c>
-      <c r="N28" s="16" t="n">
-        <v>5357.584152856845</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="inlineStr">
+      <c r="B28" s="25" t="n"/>
+      <c r="C28" s="25" t="inlineStr">
         <is>
           <t>Δ</t>
         </is>
       </c>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="26" t="n">
+      <c r="D28" s="25" t="n"/>
+      <c r="E28" s="25" t="n"/>
+      <c r="F28" s="26" t="n">
         <v>2807</v>
       </c>
-      <c r="G29" s="25" t="n"/>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
-      <c r="J29" s="25" t="n"/>
-      <c r="K29" s="26" t="n">
+      <c r="G28" s="25" t="n"/>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
+      <c r="J28" s="25" t="n"/>
+      <c r="K28" s="26" t="n">
         <v>3110.156000000003</v>
       </c>
-      <c r="L29" s="26" t="n">
+      <c r="L28" s="26" t="n">
         <v>60.56283895131457</v>
       </c>
-      <c r="M29" s="26" t="n">
+      <c r="M28" s="26" t="n">
         <v>60.56283895131463</v>
       </c>
-      <c r="N29" s="26" t="n">
+      <c r="N28" s="26" t="n">
         <v>523.6143370788777</v>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="14" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>Rule: cheapest solid = lowest estimated out-the-door figure among live cars with a verified 1-owner / 0-accident history (or Mazda CPO) at a franchise dealer; stretch = best-value live 2023 in the Turbo / Premium tiers, ranked by list price against KBB Seattle fair purchase price.</t>
         </is>
@@ -3817,7 +3667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O8"/>
+  <dimension ref="B1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -3995,75 +3845,75 @@
     </row>
     <row r="6">
       <c r="B6" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Carbon Edition</t>
+          <t>2.5 S Preferred AWD</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>CarMax Sacramento South</t>
+          <t>Royal Moore Mazda</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Hillsboro, OR</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>24998</v>
+        <v>26900</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>48337</v>
+        <v>16615</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Aug 11</t>
+          <t>Aug 13</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>Aug 11 PM</t>
+          <t>dealer email Aug 13</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>https://www.carmax.com/car/70056694</t>
+          <t>https://www.cargurus.com/Cars/listing/454567468</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Grand Touring AWD</t>
+          <t>Carbon Edition</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Doug's Lynnwood Mazda</t>
+          <t>CarMax Sacramento South</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Edmonds, WA</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="G7" s="9" t="n">
-        <v>28700</v>
+        <v>24998</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>27089</v>
+        <v>48337</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
@@ -4072,54 +3922,98 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>dealer email Aug 11 (sold Aug 10)</t>
+          <t>Aug 11 PM</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/495a1e58-37a7-480b-9f80-8bb411d8fa8f/</t>
+          <t>https://www.carmax.com/car/70056694</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Grand Touring AWD</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Doug's Lynnwood Mazda</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Edmonds, WA</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>28700</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>27089</v>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Aug 11</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>dealer email Aug 11 (sold Aug 10)</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cars.com/vehicledetail/495a1e58-37a7-480b-9f80-8bb411d8fa8f/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C9" s="8" t="n">
         <v>2023</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>2.5 S Preferred AWD</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Auto Connections of Bellevue (independent)</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G9" s="9" t="n">
         <v>26495</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>20533</v>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>Aug 11</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>Aug 11, 11:51 AM</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>https://www.cargurus.com/Cars/listing/450670232</t>
         </is>
@@ -5466,7 +5360,7 @@
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Board: Titus-Will confirmed their best number and is off the weekend visit list
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O26"/>
+  <dimension ref="B1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,7 @@
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Published Aug 7, 2026; refreshed Aug 13, 2026. Generated from data/board.json by tools/build_site.py — same rows as the web page.</t>
+          <t>Published Aug 7, 2026; refreshed Aug 14, 2026. Generated from data/board.json by tools/build_site.py — same rows as the web page.</t>
         </is>
       </c>
     </row>
@@ -604,103 +604,110 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
+          <t>Aug 14, 2026: Titus-Will: dealer confirmed their best number and stood down; the Olympia car is off the weekend visit list.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
+          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
+          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
+          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
+          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -751,7 +758,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Board — cars in play as of Aug 13, 2026 (sold cars on their own tab)</t>
+          <t>Board — cars in play as of Aug 14, 2026 (sold cars on their own tab)</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -1783,7 +1790,7 @@
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>dealer asking to schedule a Saturday time (Aug 12 evening); paperwork requested first.</t>
+          <t>dealer confirmed their best number Fri Aug 14 and left the door open; not on this weekend's visit list.</t>
         </is>
       </c>
       <c r="Y12" s="3" t="inlineStr">
@@ -4055,7 +4062,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Watchlist: screened, not on the board (re-checked Aug 13, 2026)</t>
+          <t>Watchlist: screened, not on the board (re-checked Aug 14, 2026)</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -4916,7 +4923,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>KBB fair purchase price vs. lowest clean live listing (Aug 13, 2026)</t>
+          <t>KBB fair purchase price vs. lowest clean live listing (Aug 14, 2026)</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>

</xml_diff>

<commit_message>
Board: certified 2023 Carbon worksheet received; quote recorded
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O27"/>
+  <dimension ref="B1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>15 cars in play (14 live + benchmark), 6 sold since publication, 6 written quotes in hand.</t>
+          <t>15 cars in play (14 live + benchmark), 6 sold since publication, 7 written quotes in hand.</t>
         </is>
       </c>
     </row>
@@ -604,110 +604,117 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 14, 2026: Titus-Will: dealer confirmed their best number and stood down; the Olympia car is off the weekend visit list.</t>
+          <t>Aug 14, 2026: Puyallup Mazda: itemized worksheet received for the certified 2023 Carbon (#9); zero add-ons.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
+          <t>Aug 14, 2026: Titus-Will: dealer confirmed their best number and stood down; the Olympia car is off the weekend visit list.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
+          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
+          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
+          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
+          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -1498,7 +1505,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>CPO pricing breakdown received Thu Aug 13 early afternoon; itemized worksheet attached in the dealer's email.</t>
+          <t>itemized written worksheet received Fri Aug 14; zero add-ons and the selling price came in under the advertised figure.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Correct car #5: the CARFAX shows an accident reported 7/31/2021
The full report, pulled by Hyundai of Kirkland on 8/11 and read today,
records an accident on 7/31/2021 with no airbag deployment. The car was
carried here as accident-free on the strength of a CarGurus badge. Also
captures the one-owner Washington history, 12 Doug's Lynnwood service
records, the 6/9/2026 lot date and the expired factory warranty.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -1165,7 +1165,7 @@
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 0 accidents</t>
+          <t>1 owner · 1 accident</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>updated written proposal received Thu Aug 13 midday; license billed at actuals with any overage refunded and two keys confirmed in writing; window sticker being pulled to confirm the GT Premium package; replied Thu afternoon.</t>
+          <t>CARFAX read in full Sat Aug 15: one owner, Washington only, 12 dealer service records and no open recalls, but an accident reported 7/31/2021 with no severity, no impact location and no repair record. Previously carried here as accident-free, which was wrong.</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>#5 2021 Grand Touring AWD · Hyundai of Kirkland</t>
+          <t>#4 2021 Carbon Edition Turbo · Ron Tonkin Honda</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -3577,23 +3577,23 @@
         </is>
       </c>
       <c r="F26" s="16" t="n">
-        <v>25192</v>
+        <v>25852</v>
       </c>
       <c r="G26" s="7" t="n"/>
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="16" t="n">
-        <v>28712.736</v>
+        <v>29558.646</v>
       </c>
       <c r="L26" s="16" t="n">
-        <v>559.1117635962995</v>
+        <v>575.5838348034372</v>
       </c>
       <c r="M26" s="16" t="n">
-        <v>461.7487391188865</v>
+        <v>478.2208103260242</v>
       </c>
       <c r="N26" s="16" t="n">
-        <v>4833.969815777968</v>
+        <v>4976.384088206229</v>
       </c>
     </row>
     <row r="27">
@@ -3643,23 +3643,23 @@
       <c r="D28" s="25" t="n"/>
       <c r="E28" s="25" t="n"/>
       <c r="F28" s="26" t="n">
-        <v>2807</v>
+        <v>2147</v>
       </c>
       <c r="G28" s="25" t="n"/>
       <c r="H28" s="25" t="n"/>
       <c r="I28" s="25" t="n"/>
       <c r="J28" s="25" t="n"/>
       <c r="K28" s="26" t="n">
-        <v>3110.156000000003</v>
+        <v>2264.246000000003</v>
       </c>
       <c r="L28" s="26" t="n">
-        <v>60.56283895131457</v>
+        <v>44.0907677441769</v>
       </c>
       <c r="M28" s="26" t="n">
-        <v>60.56283895131463</v>
+        <v>44.09076774417696</v>
       </c>
       <c r="N28" s="26" t="n">
-        <v>523.6143370788777</v>
+        <v>381.2000646506167</v>
       </c>
     </row>
     <row r="30">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Record the confirmed GT Premium window sheet, the scratch and the no-start
The package is confirmed in person: ventilated fronts, heated rears,
heated wheel, Active Driving Display, power folding mirrors, wiper
de-icer, rear camera only. Also records the right front bumper scratch
and the failed start that sent the car into the dealer's shop.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -1201,12 +1201,12 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>CARFAX read in full Sat Aug 15: one owner, Washington only, 12 dealer service records and no open recalls, but an accident reported 7/31/2021 with no severity, no impact location and no repair record. Previously carried here as accident-free, which was wrong.</t>
+          <t>Seen in person Sat Aug 15. The GT Premium package is confirmed on the dealer window sheet. The car did not start during the visit, the dealer suspects the battery and took it into their shop, so no test drive happened. Price discussion continuing by phone.</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>Leather, Bose, moonroof; GT Premium pkg adds ventilated fronts, heated rears + wheel, HUD.</t>
+          <t>Confirmed on the window sheet: ventilated front seats, heated rear seats, heated steering wheel, Active Driving Display, power folding mirrors, wiper de-icer. Leather, Bose, moonroof. Rear camera only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ingest the Puyallup lot evidence: stickers, CARFAXes and lower posted prices
The 2023 Turbo's original Monroney confirms the full comfort package
including ventilated seats, and its CARFAX shows one owner, a personal
lease and no accidents. The red 2021 is a Canadian-market car with a
Saskatchewan safety-inspection failure recorded 8/15/2025 and no repair
record after it, so it comes off consideration. The certified 2023's
CARFAX link would not load, so its history stays marked unverified.
All three posted prices have come down.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -930,10 +930,10 @@
         <v>27990</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>28199</v>
+        <v>27919</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>27999</v>
+        <v>27719</v>
       </c>
       <c r="J4" s="9" t="n">
         <v>200</v>
@@ -997,12 +997,12 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>written itemized quote in hand (sheet dated Aug 11, surfaced Aug 12 after a phone call; the sender's group domain had gone to spam); zero add-ons.</t>
+          <t>Seen and driven Sat Aug 15. The original window sticker confirms the full comfort package including ventilated front seats, and the CARFAX shows one owner, a personal lease and no accidents.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Loaded turbo: heated leather, Bose, sunroof, 227 hp.</t>
+          <t>Confirmed on the original window sticker: ventilated front seats, heated front and rear seats, heated steering wheel, Active Driving Display, wireless charger, power folding mirrors, Bose 10-speaker, driver seat memory, moonroof. 2.5 Turbo, 227 hp on 87 octane and 256 hp on 93.</t>
         </is>
       </c>
     </row>
@@ -1236,10 +1236,10 @@
         <v>42515</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>25198</v>
+        <v>24948</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>24998</v>
+        <v>24748</v>
       </c>
       <c r="J7" s="9" t="n">
         <v>200</v>
@@ -1265,7 +1265,7 @@
       <c r="O7" s="9" t="n"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2 owners · 0 accidents</t>
+          <t>3 owners · 0 accidents</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>written itemized quote in hand (sheet dated Aug 11, surfaced Aug 12); zero add-ons.</t>
+          <t>CARFAX read in full Sat Aug 15. A Canadian-market car with a Saskatchewan safety-inspection failure recorded 8/15/2025 and no repair record after it, imported to the United States in May 2026 and sold at auction in June. Removed from consideration.</t>
         </is>
       </c>
       <c r="Y7" s="3" t="inlineStr">
@@ -1438,10 +1438,10 @@
         <v>33006</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>27699</v>
+        <v>27424</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>27499</v>
+        <v>27224</v>
       </c>
       <c r="J9" s="9" t="n">
         <v>200</v>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>itemized written worksheet received Fri Aug 14; zero add-ons and the selling price came in under the advertised figure.</t>
+          <t>Seen Sat Aug 15. The dealer CARFAX link for this vehicle would not load, so its history remains unverified.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>24998</v>
+        <v>24748</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>0.108</v>
@@ -3224,16 +3224,16 @@
     </row>
     <row r="18">
       <c r="B18" s="6" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>2022 2.5 S Premium Plus</t>
+          <t>2023 2.5 S Carbon Edition</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Titus-Will Chevrolet GMC Cadillac</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -3242,10 +3242,10 @@
         </is>
       </c>
       <c r="F18" s="9" t="n">
-        <v>27389</v>
+        <v>27224</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.102</v>
+        <v>0.108</v>
       </c>
       <c r="H18" s="9" t="n">
         <v>200</v>
@@ -3273,22 +3273,22 @@
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>est. at Olympia, WA rate</t>
+          <t>est. at Puyallup, WA rate</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>2023 2.5 S Carbon Edition</t>
+          <t>2022 2.5 S Premium Plus</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Puyallup Mazda</t>
+          <t>Titus-Will Chevrolet GMC Cadillac</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -3297,10 +3297,10 @@
         </is>
       </c>
       <c r="F19" s="9" t="n">
-        <v>27499</v>
+        <v>27389</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>0.108</v>
+        <v>0.102</v>
       </c>
       <c r="H19" s="9" t="n">
         <v>200</v>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>est. at Puyallup, WA rate</t>
+          <t>est. at Olympia, WA rate</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="F21" s="9" t="n">
-        <v>27999</v>
+        <v>27719</v>
       </c>
       <c r="G21" s="10" t="n">
         <v>0.108</v>
@@ -3614,23 +3614,23 @@
         </is>
       </c>
       <c r="F27" s="16" t="n">
-        <v>27999</v>
+        <v>27719</v>
       </c>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="16" t="n">
-        <v>31822.892</v>
+        <v>31512.652</v>
       </c>
       <c r="L27" s="16" t="n">
-        <v>619.6746025476141</v>
+        <v>613.6334216048396</v>
       </c>
       <c r="M27" s="16" t="n">
-        <v>522.3115780702011</v>
+        <v>516.2703971274266</v>
       </c>
       <c r="N27" s="16" t="n">
-        <v>5357.584152856845</v>
+        <v>5305.35329629037</v>
       </c>
     </row>
     <row r="28">
@@ -3643,23 +3643,23 @@
       <c r="D28" s="25" t="n"/>
       <c r="E28" s="25" t="n"/>
       <c r="F28" s="26" t="n">
-        <v>2147</v>
+        <v>1867</v>
       </c>
       <c r="G28" s="25" t="n"/>
       <c r="H28" s="25" t="n"/>
       <c r="I28" s="25" t="n"/>
       <c r="J28" s="25" t="n"/>
       <c r="K28" s="26" t="n">
-        <v>2264.246000000003</v>
+        <v>1954.006000000001</v>
       </c>
       <c r="L28" s="26" t="n">
-        <v>44.0907677441769</v>
+        <v>38.04958680140237</v>
       </c>
       <c r="M28" s="26" t="n">
-        <v>44.09076774417696</v>
+        <v>38.04958680140243</v>
       </c>
       <c r="N28" s="26" t="n">
-        <v>381.2000646506167</v>
+        <v>328.9692080841414</v>
       </c>
     </row>
     <row r="30">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="E7" s="9" t="n"/>
       <c r="F7" s="9" t="n">
-        <v>25198</v>
+        <v>24948</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         <v>30980</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>28199</v>
+        <v>27919</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close the search: the 2023 Turbo was purchased Aug 15
Marks VIN JM3KFBAY3P0289626 purchased, freezes the board as of that
date, and adds the closing changelog entry. Figures stay off the public
pages as always.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HSSGkNu3Mr9vQrXnxF1MKw
</commit_message>
<xml_diff>
--- a/CX5-Seattle-Buyers-Report.xlsx
+++ b/CX5-Seattle-Buyers-Report.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O28"/>
+  <dimension ref="B1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>15 cars in play (14 live + benchmark), 6 sold since publication, 7 written quotes in hand.</t>
+          <t>14 cars in play (13 live + benchmark), 7 sold since publication, 6 written quotes in hand.</t>
         </is>
       </c>
     </row>
@@ -604,117 +604,145 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Aug 14, 2026: Puyallup Mazda: itemized worksheet received for the certified 2023 Carbon (#9); zero add-ons.</t>
+          <t>Aug 15, 2026: Search closed. The buyer purchased the 2023 CX-5 2.5 Turbo AWD (VIN JM3KFBAY3P0289626, 27,990 miles) from Puyallup Mazda on Aug 15 2026.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Aug 14, 2026: Titus-Will: dealer confirmed their best number and stood down; the Olympia car is off the weekend visit list.</t>
+          <t>Aug 15, 2026: The board is frozen as of that date. Prices, availability and history notes on the remaining cars reflect the last verification before close and are no longer being maintained.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
+          <t>Aug 15, 2026: Verified in person that day: the 2023 Turbo's original window sticker (full comfort package standard on the 25T trim) and a clean one-owner CARFAX.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
+          <t>Aug 15, 2026: Removed from consideration: Puyallup's red 2021, a Canadian-market car whose CARFAX records a Saskatchewan safety-inspection failure on 8/15/2025 with no repair record after it.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
+          <t>Aug 14, 2026: Puyallup Mazda: itemized worksheet received for the certified 2023 Carbon (#9); zero add-ons.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
+          <t>Aug 14, 2026: Titus-Will: dealer confirmed their best number and stood down; the Olympia car is off the weekend visit list.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
+          <t>Aug 13, 2026: Royal Moore: one 2023 Preferred sold per the dealer; the remaining one was requoted with the dealer-added items removed.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
+          <t>Aug 13, 2026: Puyallup Mazda: pricing breakdown received for the CPO 2023 Carbon (#9); worksheet attached in email.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
+          <t>Aug 13, 2026: Royal Moore: manager follow-up received Thu afternoon; reply prepared.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
+          <t>Aug 13, 2026: Hyundai of Kirkland: updated written proposal received midday; license-at-actuals refund and two keys confirmed in writing; window sticker check in progress.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
+          <t>Aug 12, 2026: Puyallup Mazda (#1, #6): written itemized quotes surfaced (sheets dated Aug 11 had landed in spam); zero add-ons on both. #9's breakdown requested.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
+          <t>Aug 12, 2026: Lee Johnson (#7, #12): both inquiry emails bounced back undelivered (dealer mail server unreachable); a new contact path is being arranged.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+          <t>Aug 12, 2026: Fresh read-only sweep (AutoTempest, CarGurus, KBB, CarMax, Carvana, Craigslist: 386 raw / 223 VINs). Every live board car re-verified with no listed-price change; #12 (Cars.com-only) could not be re-checked from the sweep environment.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+          <t>Aug 12, 2026: 26 VINs not seen before: 25 disqualified (unwanted trim, out-of-area no-haggle units no better than #15, no value signal), 1 added as #21 (2021 Signature, Burlington WA, $25,999 + $200).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+          <t>Aug 12, 2026: Rodland (#14) pricing sheet transcribed: clean sheet, no add-ons; tax and licence lumped in one line, itemization requested.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+          <t>Aug 12, 2026: Site now regenerates every section and download from one board file, so the cost table, compare box, calculator and top picks follow the live set (sold #3 dropped from the picks; quoted OTDs replace estimates where dealers have replied).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Aug 12, 2026: 2024 model-year sweep — no verified-clean, non-rental 2024 Preferred/Carbon/Premium under 40k mi lands at or below the finalists’ $28.7–32k est. OTD; three 2024s added to the watchlist (watch only, not numbered board cars).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Buyer outreach began: itemized-OTD requests to every live dealer; written numbers back from Kirkland (#5), Titus-Will (#13, revised), Auto 206 (#17), Rodland (#14) and Royal Moore (#8, add-ons to strike).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Sold and removed: #2 Acura of Seattle Turbo, #3 BMW Seattle GT Reserve (dealer-confirmed), #11 CarMax Sacramento, #16 Doug’s Lynnwood GT, #18 Auto Connections Bellevue. #1’s reported sale was wrong (live on CarGurus and Puyallup Mazda’s own site at $27,999).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026: Comfort-first re-rank and WA-first re-scan added #12–#20; tax model corrected to dealer-city rates (Seattle 11.05%) from the flat 10.35% used on Aug 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Aug 7, 2026: Initial read-only market scan: 278 raw listings → 153 unique VINs → 112 pass the disqualifiers; 11-car shortlist ranked by value.</t>
         </is>
@@ -732,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Y18"/>
+  <dimension ref="B1:Y17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -906,7 +934,7 @@
     </row>
     <row r="4">
       <c r="B4" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
@@ -914,11 +942,11 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>2.5 Turbo AWD</t>
+          <t>Carbon Edition Turbo</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -927,37 +955,37 @@
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>27990</v>
+        <v>34800</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>27919</v>
+        <v>26102</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>27719</v>
+        <v>25852</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Puyallup Mazda</t>
+          <t>Ron Tonkin Honda</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>Puyallup, WA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="M4" s="10" t="n">
-        <v>0.108</v>
+        <v>0.1105</v>
       </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
-          <t>Great · $2,781 &lt; FPP</t>
+          <t>Great · $2,612 &lt; FPP</t>
         </is>
       </c>
       <c r="O4" s="9" t="n">
-        <v>30980</v>
+        <v>29374</v>
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
@@ -970,45 +998,45 @@
         </is>
       </c>
       <c r="R4" s="6" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="S4" s="7" t="inlineStr">
         <is>
-          <t>CarGurus</t>
+          <t>KBB</t>
         </is>
       </c>
       <c r="T4" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/448185375</t>
+          <t>https://www.kbb.com/cars-for-sale/vehicle/782577606</t>
         </is>
       </c>
       <c r="U4" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBAY3P0289626</t>
+          <t>JM3KFBCYXM0385696</t>
         </is>
       </c>
       <c r="V4" s="7" t="inlineStr">
         <is>
-          <t>YW29065</t>
+          <t>UH1679</t>
         </is>
       </c>
       <c r="W4" s="6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Seen and driven Sat Aug 15. The original window sticker confirms the full comfort package including ventilated front seats, and the CARFAX shows one owner, a personal lease and no accidents.</t>
+          <t>quote in preparation (Aug 11, 3:57 PM); our written-number request is with the dealer. Oregon: email-only leverage.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Confirmed on the original window sticker: ventilated front seats, heated front and rear seats, heated steering wheel, Active Driving Display, wireless charger, power folding mirrors, Bose 10-speaker, driver seat memory, moonroof. 2.5 Turbo, 227 hp on 87 octane and 256 hp on 93.</t>
+          <t>Carbon look, heated seats; turbo confirmed by the dealer.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
@@ -1020,50 +1048,50 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Carbon Edition Turbo</t>
+          <t>Grand Touring AWD</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>2.5 Turbo</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>34800</v>
+        <v>33336</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>26102</v>
+        <v>25192</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>25852</v>
+        <v>25192</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Ron Tonkin Honda</t>
+          <t>Hyundai of Kirkland / Ford of Kirkland</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Kirkland, WA</t>
         </is>
       </c>
       <c r="M5" s="10" t="n">
-        <v>0.1105</v>
+        <v>0.108</v>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>Great · $2,612 &lt; FPP</t>
+          <t>Good · $3,338 &lt; FPP</t>
         </is>
       </c>
       <c r="O5" s="9" t="n">
-        <v>29374</v>
+        <v>28530</v>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 0 accidents</t>
+          <t>1 owner · 1 accident</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
@@ -1072,45 +1100,45 @@
         </is>
       </c>
       <c r="R5" s="6" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>KBB</t>
+          <t>CarGurus</t>
         </is>
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>https://www.kbb.com/cars-for-sale/vehicle/782577606</t>
+          <t>https://www.cargurus.com/Cars/listing/451807182</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCYXM0385696</t>
+          <t>JM3KFBDM3M0301052</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>UH1679</t>
+          <t>O94564A</t>
         </is>
       </c>
       <c r="W5" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>quote in preparation (Aug 11, 3:57 PM); our written-number request is with the dealer. Oregon: email-only leverage.</t>
+          <t>Seen in person Sat Aug 15. The GT Premium package is confirmed on the dealer window sheet. The car did not start during the visit, the dealer suspects the battery and took it into their shop, so no test drive happened. Price discussion continuing by phone.</t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t>Carbon look, heated seats; turbo confirmed by the dealer.</t>
+          <t>Confirmed on the window sheet: ventilated front seats, heated rear seats, heated steering wheel, Active Driving Display, power folding mirrors, wiper de-icer. Leather, Bose, moonroof. Rear camera only.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
@@ -1122,34 +1150,34 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Grand Touring AWD</t>
+          <t>Carbon Ed Turbo AWD</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5 Turbo</t>
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>33336</v>
+        <v>42515</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>25192</v>
+        <v>24948</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>25192</v>
+        <v>24748</v>
       </c>
       <c r="J6" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Hyundai of Kirkland / Ford of Kirkland</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>Kirkland, WA</t>
+          <t>Puyallup, WA</t>
         </is>
       </c>
       <c r="M6" s="10" t="n">
@@ -1157,15 +1185,13 @@
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>Good · $3,338 &lt; FPP</t>
-        </is>
-      </c>
-      <c r="O6" s="9" t="n">
-        <v>28530</v>
-      </c>
+          <t>Great · $1,939 below</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="n"/>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 1 accident</t>
+          <t>3 owners · 0 accidents</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
@@ -1174,7 +1200,7 @@
         </is>
       </c>
       <c r="R6" s="6" t="n">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="S6" s="7" t="inlineStr">
         <is>
@@ -1183,36 +1209,36 @@
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/451807182</t>
+          <t>https://www.cargurus.com/Cars/listing/449972241</t>
         </is>
       </c>
       <c r="U6" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM3M0301052</t>
+          <t>JM3KFBDYXM0120596</t>
         </is>
       </c>
       <c r="V6" s="7" t="inlineStr">
         <is>
-          <t>O94564A</t>
+          <t>YS29241</t>
         </is>
       </c>
       <c r="W6" s="6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>Seen in person Sat Aug 15. The GT Premium package is confirmed on the dealer window sheet. The car did not start during the visit, the dealer suspects the battery and took it into their shop, so no test drive happened. Price discussion continuing by phone.</t>
+          <t>CARFAX read in full Sat Aug 15. A Canadian-market car with a Saskatchewan safety-inspection failure recorded 8/15/2025 and no repair record after it, imported to the United States in May 2026 and sold at auction in June. Removed from consideration.</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>Confirmed on the window sheet: ventilated front seats, heated rear seats, heated steering wheel, Active Driving Display, power folding mirrors, wiper de-icer. Leather, Bose, moonroof. Rear camera only.</t>
+          <t>Carbon look: Soul Red, black 19s, heated seats, turbo.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
@@ -1220,61 +1246,63 @@
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Carbon Ed Turbo AWD</t>
+          <t>2.5 S Carbon Edition</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>2.5 Turbo</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>42515</v>
+        <v>34749</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>24948</v>
+        <v>27512</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>24748</v>
+        <v>27512</v>
       </c>
       <c r="J7" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Puyallup Mazda</t>
+          <t>Lee Johnson Mazda of Seattle</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>Puyallup, WA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="M7" s="10" t="n">
-        <v>0.108</v>
+        <v>0.1105</v>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>Great · $1,939 below</t>
-        </is>
-      </c>
-      <c r="O7" s="9" t="n"/>
+          <t>Good · $349 below</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>27440</v>
+      </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>3 owners · 0 accidents</t>
+          <t>1 owner · 0 accidents</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R7" s="6" t="n">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="S7" s="7" t="inlineStr">
         <is>
@@ -1283,36 +1311,36 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/449972241</t>
+          <t>https://www.cargurus.com/Cars/listing/453287059</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDYXM0120596</t>
+          <t>JM3KFBCM4N0546820</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>YS29241</t>
+          <t>U14590</t>
         </is>
       </c>
       <c r="W7" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>CARFAX read in full Sat Aug 15. A Canadian-market car with a Saskatchewan safety-inspection failure recorded 8/15/2025 and no repair record after it, imported to the United States in May 2026 and sold at auction in June. Removed from consideration.</t>
+          <t>two-car OTD request emailed Aug 11 — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
         </is>
       </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>Carbon look: Soul Red, black 19s, heated seats, turbo.</t>
+          <t>Red leather, heated fronts, moonroof, Mazda CPO warranty.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
@@ -1320,7 +1348,7 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -1333,37 +1361,37 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>34749</v>
+        <v>33006</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>27512</v>
+        <v>27424</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>27512</v>
+        <v>27224</v>
       </c>
       <c r="J8" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Lee Johnson Mazda of Seattle</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Puyallup, WA</t>
         </is>
       </c>
       <c r="M8" s="10" t="n">
-        <v>0.1105</v>
+        <v>0.108</v>
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>Good · $349 below</t>
+          <t>Good · $518 below</t>
         </is>
       </c>
       <c r="O8" s="9" t="n">
-        <v>27440</v>
+        <v>28090</v>
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
@@ -1376,7 +1404,7 @@
         </is>
       </c>
       <c r="R8" s="6" t="n">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="S8" s="7" t="inlineStr">
         <is>
@@ -1385,36 +1413,36 @@
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/453287059</t>
+          <t>https://www.cargurus.com/Cars/listing/450917825</t>
         </is>
       </c>
       <c r="U8" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCM4N0546820</t>
+          <t>JM3KFBCMXP0288130</t>
         </is>
       </c>
       <c r="V8" s="7" t="inlineStr">
         <is>
-          <t>U14590</t>
+          <t>M260362A</t>
         </is>
       </c>
       <c r="W8" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>two-car OTD request emailed Aug 11 — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
+          <t>Seen Sat Aug 15. The dealer CARFAX link for this vehicle would not load, so its history remains unverified.</t>
         </is>
       </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>Red leather, heated fronts, moonroof, Mazda CPO warranty.</t>
+          <t>Red leather, heated fronts, Mazda CPO warranty.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
@@ -1426,7 +1454,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Carbon Edition</t>
+          <t>2.5 S Preferred</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1435,88 +1463,86 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>33006</v>
+        <v>44989</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>27424</v>
+        <v>24095</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>27224</v>
+        <v>23995</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Puyallup Mazda</t>
+          <t>Columbia Sales &amp; Service</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Puyallup, WA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="M9" s="10" t="n">
-        <v>0.108</v>
+        <v>0.1105</v>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>Good · $518 below</t>
-        </is>
-      </c>
-      <c r="O9" s="9" t="n">
-        <v>28090</v>
-      </c>
+          <t>Great · Cars.com rating</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="n"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 0 accidents</t>
+          <t>2 owners · 0 accidents</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R9" s="6" t="n">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>CarGurus</t>
+          <t>Cars.com</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/450917825</t>
+          <t>https://www.cars.com/vehicledetail/d4fd9d01-99f9-4673-87c0-1a173ef9551f/</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCMXP0288130</t>
+          <t>JM3KFBCM9P0119426</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>M260362A</t>
+          <t>2468</t>
         </is>
       </c>
       <c r="W9" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>Seen Sat Aug 15. The dealer CARFAX link for this vehicle would not load, so its history remains unverified.</t>
+          <t>emailed Aug 11, no reply. Oregon: email-only.</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t>Red leather, heated fronts, Mazda CPO warranty.</t>
+          <t>Leatherette, heated fronts, moonroof.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
@@ -1528,7 +1554,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred</t>
+          <t>2.5 S Preferred · Mazda CPO</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1537,49 +1563,43 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>44989</v>
+        <v>36400</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>24095</v>
+        <v>26348</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>23995</v>
+        <v>26348</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Columbia Sales &amp; Service</t>
+          <t>Lee Johnson Mazda of Seattle</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="M10" s="10" t="n">
         <v>0.1105</v>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>Great · Cars.com rating</t>
-        </is>
-      </c>
+      <c r="N10" s="7" t="inlineStr"/>
       <c r="O10" s="9" t="n"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>2 owners · 0 accidents</t>
+          <t>0 accidents</t>
         </is>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="R10" s="6" t="n">
-        <v>29</v>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R10" s="6" t="n"/>
       <c r="S10" s="7" t="inlineStr">
         <is>
           <t>Cars.com</t>
@@ -1587,36 +1607,32 @@
       </c>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/d4fd9d01-99f9-4673-87c0-1a173ef9551f/</t>
+          <t>https://www.cars.com/vehicledetail/d7b0a899-fdc8-4776-9379-64684c757f41/</t>
         </is>
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCM9P0119426</t>
-        </is>
-      </c>
-      <c r="V10" s="7" t="inlineStr">
-        <is>
-          <t>2468</t>
-        </is>
-      </c>
+          <t>JM3KFBCM7P0256994</t>
+        </is>
+      </c>
+      <c r="V10" s="7" t="n"/>
       <c r="W10" s="6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>emailed Aug 11, no reply. Oregon: email-only.</t>
+          <t>in the Lee Johnson two-car OTD request (Aug 11) — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
-          <t>Leatherette, heated fronts, moonroof.</t>
+          <t>Leather-trimmed Preferred content (heated fronts, moonroof) with the Mazda CPO warranty.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
@@ -1624,11 +1640,11 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred · Mazda CPO</t>
+          <t>2.5 S Premium Plus</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1637,76 +1653,88 @@
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>36400</v>
+        <v>43640</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>26348</v>
+        <v>27389</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>26348</v>
+        <v>27389</v>
       </c>
       <c r="J11" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Lee Johnson Mazda of Seattle</t>
+          <t>Titus-Will Chevrolet GMC Cadillac</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Olympia, WA</t>
         </is>
       </c>
       <c r="M11" s="10" t="n">
-        <v>0.1105</v>
-      </c>
-      <c r="N11" s="7" t="inlineStr"/>
-      <c r="O11" s="9" t="n"/>
+        <v>0.102</v>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>Good · $389 over FPP</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>27000</v>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>0 accidents</t>
+          <t>1 owner · 0 accidents</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="R11" s="6" t="n"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>45</v>
+      </c>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Cars.com</t>
+          <t>KBB</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/d7b0a899-fdc8-4776-9379-64684c757f41/</t>
+          <t>https://www.kbb.com/cars-for-sale/vehicle/784195725</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBCM7P0256994</t>
-        </is>
-      </c>
-      <c r="V11" s="7" t="n"/>
+          <t>JM3KFBEM1N0590576</t>
+        </is>
+      </c>
+      <c r="V11" s="7" t="inlineStr">
+        <is>
+          <t>P11101</t>
+        </is>
+      </c>
       <c r="W11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>in the Lee Johnson two-car OTD request (Aug 11) — both emails to the dealer's listed sales address bounced back Aug 12 (server unreachable after 24h of retries) — the request never arrived; a new contact path is being arranged.</t>
+          <t>dealer confirmed their best number Fri Aug 14 and left the door open; not on this weekend's visit list.</t>
         </is>
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>Leather-trimmed Preferred content (heated fronts, moonroof) with the Mazda CPO warranty.</t>
+          <t>Ventilated seats, HUD, heated rears; CarBravo (GM) certified, not Mazda CPO.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
@@ -1714,11 +1742,11 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Premium Plus</t>
+          <t>2.5 S Premium</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1727,37 +1755,37 @@
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>43640</v>
+        <v>17505</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>27389</v>
+        <v>28487</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>27389</v>
+        <v>28287</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Titus-Will Chevrolet GMC Cadillac</t>
+          <t>Rodland Toyota of Everett</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>Olympia, WA</t>
+          <t>Everett, WA</t>
         </is>
       </c>
       <c r="M12" s="10" t="n">
-        <v>0.102</v>
+        <v>0.104</v>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>Good · $389 over FPP</t>
+          <t>Good · $873 below</t>
         </is>
       </c>
       <c r="O12" s="9" t="n">
-        <v>27000</v>
+        <v>27750</v>
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
@@ -1770,49 +1798,49 @@
         </is>
       </c>
       <c r="R12" s="6" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="S12" s="7" t="inlineStr">
         <is>
-          <t>KBB</t>
+          <t>CarGurus</t>
         </is>
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>https://www.kbb.com/cars-for-sale/vehicle/784195725</t>
+          <t>https://www.cargurus.com/Cars/listing/453332129</t>
         </is>
       </c>
       <c r="U12" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBEM1N0590576</t>
+          <t>JM3KFBDM7P0281828</t>
         </is>
       </c>
       <c r="V12" s="7" t="inlineStr">
         <is>
-          <t>P11101</t>
+          <t>68987A</t>
         </is>
       </c>
       <c r="W12" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>dealer confirmed their best number Fri Aug 14 and left the door open; not on this weekend's visit list.</t>
+          <t>dealer declined to negotiate by email (Aug 12 evening); no visit planned.</t>
         </is>
       </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>Ventilated seats, HUD, heated rears; CarBravo (GM) certified, not Mazda CPO.</t>
+          <t>Lowest-mile comfort car in the set: Soul Red, leather, Bose, heated wheel (no ventilation).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
@@ -1820,7 +1848,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Premium</t>
+          <t>2.5 S Premium · no-haggle</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1829,38 +1857,36 @@
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>17505</v>
+        <v>31166</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>28487</v>
+        <v>27998</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>28287</v>
+        <v>27998</v>
       </c>
       <c r="J13" s="9" t="n">
         <v>200</v>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Rodland Toyota of Everett</t>
+          <t>CarMax Renton</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>Everett, WA</t>
+          <t>Renton, WA</t>
         </is>
       </c>
       <c r="M13" s="10" t="n">
-        <v>0.104</v>
+        <v>0.11</v>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>Good · $873 below</t>
-        </is>
-      </c>
-      <c r="O13" s="9" t="n">
-        <v>27750</v>
-      </c>
+          <t>Fair · $222 below</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="n"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
           <t>1 owner · 0 accidents</t>
@@ -1872,57 +1898,57 @@
         </is>
       </c>
       <c r="R13" s="6" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>CarGurus</t>
+          <t>CarMax</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/453332129</t>
+          <t>https://www.cargurus.com/Cars/listing/455754266</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM7P0281828</t>
+          <t>JM3KFBDM0P0215315</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>68987A</t>
+          <t>70134808</t>
         </is>
       </c>
       <c r="W13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>dealer declined to negotiate by email (Aug 12 evening); no visit planned.</t>
+          <t>reference car; nothing to request.</t>
         </is>
       </c>
       <c r="Y13" s="3" t="inlineStr">
         <is>
-          <t>Lowest-mile comfort car in the set: Soul Red, leather, Bose, heated wheel (no ventilation).</t>
+          <t>In-state no-haggle benchmark, no transfer fee.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>benchmark</t>
+          <t>live</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Premium · no-haggle</t>
+          <t>Grand Touring w/ GT Premium pkg</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -1931,39 +1957,41 @@
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>31166</v>
+        <v>30066</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>27998</v>
+        <v>25799</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>27998</v>
+        <v>25799</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>CarMax Renton</t>
+          <t>Auto 206 (independent)</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>Renton, WA</t>
+          <t>Kent, WA</t>
         </is>
       </c>
       <c r="M14" s="10" t="n">
-        <v>0.11</v>
+        <v>0.109</v>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>Fair · $222 below</t>
-        </is>
-      </c>
-      <c r="O14" s="9" t="n"/>
+          <t>$3,281 &lt; FPP</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="n">
+        <v>29080</v>
+      </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 0 accidents</t>
+          <t>1 owner · 1 accident</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
@@ -1972,45 +2000,43 @@
         </is>
       </c>
       <c r="R14" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S14" s="7" t="inlineStr">
         <is>
-          <t>CarMax</t>
+          <t>Autotrader</t>
         </is>
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/455754266</t>
+          <t>https://www.autotrader.com/cars-for-sale/vehicle/787629893</t>
         </is>
       </c>
       <c r="U14" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM0P0215315</t>
+          <t>JM3KFBDM0M0305902</t>
         </is>
       </c>
       <c r="V14" s="7" t="inlineStr">
         <is>
-          <t>70134808</t>
-        </is>
-      </c>
-      <c r="W14" s="6" t="n">
-        <v>6</v>
-      </c>
+          <t>13014</t>
+        </is>
+      </c>
+      <c r="W14" s="6" t="n"/>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>reference car; nothing to request.</t>
+          <t>written offer in hand, valid to Aug 12, 7 PM; Carfax shows a 6/2024 accident. Discussion paused.</t>
         </is>
       </c>
       <c r="Y14" s="3" t="inlineStr">
         <is>
-          <t>In-state no-haggle benchmark, no transfer fee.</t>
+          <t>Ventilated seats at GT money (GT Premium package), Deep Crystal Blue.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
@@ -2022,50 +2048,50 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Grand Touring w/ GT Premium pkg</t>
+          <t>Signature (2.5T, ventilated)</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5 Turbo</t>
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>30066</v>
+        <v>40451</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>25799</v>
+        <v>26712</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>25799</v>
+        <v>26712</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>Auto 206 (independent)</t>
+          <t>Tonkin Gresham Honda</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>Kent, WA</t>
+          <t>Troutdale, OR</t>
         </is>
       </c>
       <c r="M15" s="10" t="n">
-        <v>0.109</v>
+        <v>0.1105</v>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>$3,281 &lt; FPP</t>
+          <t>Good · $700 below</t>
         </is>
       </c>
       <c r="O15" s="9" t="n">
-        <v>29080</v>
+        <v>24480</v>
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>1 owner · 1 accident</t>
+          <t>2 owners · 0 accidents</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
@@ -2074,43 +2100,43 @@
         </is>
       </c>
       <c r="R15" s="6" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Autotrader</t>
+          <t>Cars.com</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>https://www.autotrader.com/cars-for-sale/vehicle/787629893</t>
+          <t>https://www.cars.com/vehicledetail/671f18d1-7917-4929-b9c7-3f175ba4013f/</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>JM3KFBDM0M0305902</t>
+          <t>JM3KFBEY2M0349546</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>13014</t>
+          <t>G6186020B</t>
         </is>
       </c>
       <c r="W15" s="6" t="n"/>
       <c r="X15" s="3" t="inlineStr">
         <is>
-          <t>written offer in hand, valid to Aug 12, 7 PM; Carfax shows a 6/2024 accident. Discussion paused.</t>
+          <t>not contacted; Oregon fallback, email-only.</t>
         </is>
       </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
-          <t>Ventilated seats at GT money (GT Premium package), Deep Crystal Blue.</t>
+          <t>Top 2021 trim (Nappa, vents, 360 camera).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
@@ -2118,54 +2144,48 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Signature (2.5T, ventilated)</t>
+          <t>2.5 S Preferred</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>2.5 Turbo</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>40451</v>
+        <v>16969</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>26712</v>
+        <v>26500</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>26712</v>
+        <v>26500</v>
       </c>
       <c r="J16" s="9" t="n">
         <v>250</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Tonkin Gresham Honda</t>
+          <t>Royal Moore Mazda</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>Troutdale, OR</t>
+          <t>Hillsboro, OR</t>
         </is>
       </c>
       <c r="M16" s="10" t="n">
         <v>0.1105</v>
       </c>
-      <c r="N16" s="7" t="inlineStr">
-        <is>
-          <t>Good · $700 below</t>
-        </is>
-      </c>
-      <c r="O16" s="9" t="n">
-        <v>24480</v>
-      </c>
+      <c r="N16" s="7" t="inlineStr"/>
+      <c r="O16" s="9" t="n"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>2 owners · 0 accidents</t>
+          <t>0 accidents</t>
         </is>
       </c>
       <c r="Q16" s="7" t="inlineStr">
@@ -2183,34 +2203,26 @@
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/671f18d1-7917-4929-b9c7-3f175ba4013f/</t>
-        </is>
-      </c>
-      <c r="U16" s="7" t="inlineStr">
-        <is>
-          <t>JM3KFBEY2M0349546</t>
-        </is>
-      </c>
-      <c r="V16" s="7" t="inlineStr">
-        <is>
-          <t>G6186020B</t>
-        </is>
-      </c>
+          <t>https://www.cars.com/vehicledetail/84b6552a-4a94-4c5b-96bf-0b3b37cc55a9/</t>
+        </is>
+      </c>
+      <c r="U16" s="7" t="n"/>
+      <c r="V16" s="7" t="n"/>
       <c r="W16" s="6" t="n"/>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>not contacted; Oregon fallback, email-only.</t>
+          <t>dealer requoted their remaining 2023 Preferred (stock p12315) Thu Aug 13 with the dealer-added items removed.</t>
         </is>
       </c>
       <c r="Y16" s="3" t="inlineStr">
         <is>
-          <t>Top 2021 trim (Nappa, vents, 360 camera).</t>
+          <t>The Royal Moore group's second low-mile Preferred (Toyota store, same auto center as #8).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -2218,48 +2230,54 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred</t>
+          <t>Signature (2.5T)</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5 Turbo</t>
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>16969</v>
+        <v>35589</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>26500</v>
+        <v>25999</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>26500</v>
+        <v>25999</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>Royal Moore Mazda</t>
+          <t>Cortes Auto Center (independent)</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Hillsboro, OR</t>
+          <t>Burlington, WA</t>
         </is>
       </c>
       <c r="M17" s="10" t="n">
-        <v>0.1105</v>
-      </c>
-      <c r="N17" s="7" t="inlineStr"/>
-      <c r="O17" s="9" t="n"/>
+        <v>0.091</v>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>Good · $789 over FPP</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="n">
+        <v>25410</v>
+      </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>0 accidents</t>
+          <t>1 owner · 0 accidents</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
@@ -2268,127 +2286,35 @@
         </is>
       </c>
       <c r="R17" s="6" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Cars.com</t>
+          <t>KBB</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/84b6552a-4a94-4c5b-96bf-0b3b37cc55a9/</t>
-        </is>
-      </c>
-      <c r="U17" s="7" t="n"/>
-      <c r="V17" s="7" t="n"/>
+          <t>https://www.kbb.com/cars-for-sale/vehicle/787933636</t>
+        </is>
+      </c>
+      <c r="U17" s="7" t="inlineStr">
+        <is>
+          <t>JM3KFBEY0M0417715</t>
+        </is>
+      </c>
+      <c r="V17" s="7" t="inlineStr">
+        <is>
+          <t>B1851</t>
+        </is>
+      </c>
       <c r="W17" s="6" t="n"/>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t>dealer requoted their remaining 2023 Preferred (stock p12315) Thu Aug 13 with the dealer-added items removed.</t>
+          <t>not contacted (found Aug 12).</t>
         </is>
       </c>
       <c r="Y17" s="3" t="inlineStr">
-        <is>
-          <t>The Royal Moore group's second low-mile Preferred (Toyota store, same auto center as #8).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Signature (2.5T)</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>2.5 Turbo</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>35589</v>
-      </c>
-      <c r="H18" s="9" t="n">
-        <v>25999</v>
-      </c>
-      <c r="I18" s="9" t="n">
-        <v>25999</v>
-      </c>
-      <c r="J18" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="K18" s="7" t="inlineStr">
-        <is>
-          <t>Cortes Auto Center (independent)</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>Burlington, WA</t>
-        </is>
-      </c>
-      <c r="M18" s="10" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>Good · $789 over FPP</t>
-        </is>
-      </c>
-      <c r="O18" s="9" t="n">
-        <v>25410</v>
-      </c>
-      <c r="P18" s="7" t="inlineStr">
-        <is>
-          <t>1 owner · 0 accidents</t>
-        </is>
-      </c>
-      <c r="Q18" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="R18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="7" t="inlineStr">
-        <is>
-          <t>KBB</t>
-        </is>
-      </c>
-      <c r="T18" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kbb.com/cars-for-sale/vehicle/787933636</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="inlineStr">
-        <is>
-          <t>JM3KFBEY0M0417715</t>
-        </is>
-      </c>
-      <c r="V18" s="7" t="inlineStr">
-        <is>
-          <t>B1851</t>
-        </is>
-      </c>
-      <c r="W18" s="6" t="n"/>
-      <c r="X18" s="3" t="inlineStr">
-        <is>
-          <t>not contacted (found Aug 12).</t>
-        </is>
-      </c>
-      <c r="Y18" s="3" t="inlineStr">
         <is>
           <t>WA car, top 2021 trim (Nappa leather, ventilated fronts, 360 camera, turbo), Snowflake White / Caturra Brown.</t>
         </is>
@@ -2561,7 +2487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O30"/>
+  <dimension ref="B1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -3388,187 +3314,169 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>2023 2.5 Turbo AWD</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Puyallup Mazda</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="B21" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>2023 2.5 S Premium · no-haggle (benchmark)</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>CarMax Renton</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
-      <c r="F21" s="9" t="n">
-        <v>27719</v>
-      </c>
-      <c r="G21" s="10" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="H21" s="9" t="n">
+      <c r="F21" s="20" t="n">
+        <v>27998</v>
+      </c>
+      <c r="G21" s="21" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H21" s="20" t="n">
         <v>200</v>
       </c>
-      <c r="I21" s="16">
+      <c r="I21" s="22">
         <f>F21*(1+G21)+H21+$C$6</f>
         <v/>
       </c>
-      <c r="J21" s="17" t="n"/>
-      <c r="K21" s="12">
+      <c r="J21" s="23" t="n"/>
+      <c r="K21" s="24">
         <f>IF(J21&gt;0,J21,I21)</f>
         <v/>
       </c>
-      <c r="L21" s="16">
+      <c r="L21" s="22">
         <f>-PMT($C$3/12,$C$4,K21)</f>
         <v/>
       </c>
-      <c r="M21" s="16">
+      <c r="M21" s="22">
         <f>-PMT($C$3/12,$C$4,MAX(0,K21-$C$5))</f>
         <v/>
       </c>
-      <c r="N21" s="16">
+      <c r="N21" s="22">
         <f>L21*$C$4-K21</f>
         <v/>
       </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>est. at Puyallup, WA rate</t>
+      <c r="O21" s="19" t="inlineStr">
+        <is>
+          <t>est. at Renton, WA rate</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>2023 2.5 S Premium · no-haggle (benchmark)</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>CarMax Renton</t>
-        </is>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="B22" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>2023 2.5 S Premium</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Rodland Toyota of Everett</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
-      <c r="F22" s="20" t="n">
-        <v>27998</v>
-      </c>
-      <c r="G22" s="21" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="H22" s="20" t="n">
+      <c r="F22" s="9" t="n">
+        <v>28287</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="H22" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="16">
         <f>F22*(1+G22)+H22+$C$6</f>
         <v/>
       </c>
-      <c r="J22" s="23" t="n"/>
-      <c r="K22" s="24">
+      <c r="J22" s="17" t="n"/>
+      <c r="K22" s="12">
         <f>IF(J22&gt;0,J22,I22)</f>
         <v/>
       </c>
-      <c r="L22" s="22">
+      <c r="L22" s="16">
         <f>-PMT($C$3/12,$C$4,K22)</f>
         <v/>
       </c>
-      <c r="M22" s="22">
+      <c r="M22" s="16">
         <f>-PMT($C$3/12,$C$4,MAX(0,K22-$C$5))</f>
         <v/>
       </c>
-      <c r="N22" s="22">
+      <c r="N22" s="16">
         <f>L22*$C$4-K22</f>
         <v/>
       </c>
-      <c r="O22" s="19" t="inlineStr">
-        <is>
-          <t>est. at Renton, WA rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>2023 2.5 S Premium</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Rodland Toyota of Everett</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>est. at Everett, WA rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Cheapest solid vs. stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Cheapest solid</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>#4 2021 Carbon Edition Turbo · Ron Tonkin Honda</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
-      <c r="F23" s="9" t="n">
-        <v>28287</v>
-      </c>
-      <c r="G23" s="10" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I23" s="16">
-        <f>F23*(1+G23)+H23+$C$6</f>
-        <v/>
-      </c>
-      <c r="J23" s="17" t="n"/>
-      <c r="K23" s="12">
-        <f>IF(J23&gt;0,J23,I23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="16">
-        <f>-PMT($C$3/12,$C$4,K23)</f>
-        <v/>
-      </c>
-      <c r="M23" s="16">
-        <f>-PMT($C$3/12,$C$4,MAX(0,K23-$C$5))</f>
-        <v/>
-      </c>
-      <c r="N23" s="16">
-        <f>L23*$C$4-K23</f>
-        <v/>
-      </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>est. at Everett, WA rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Cheapest solid vs. stretch</t>
-        </is>
+      <c r="F25" s="16" t="n">
+        <v>25852</v>
+      </c>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="16" t="n">
+        <v>29558.646</v>
+      </c>
+      <c r="L25" s="16" t="n">
+        <v>575.5838348034372</v>
+      </c>
+      <c r="M25" s="16" t="n">
+        <v>478.2208103260242</v>
+      </c>
+      <c r="N25" s="16" t="n">
+        <v>4976.384088206229</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Cheapest solid</t>
+          <t>Stretch</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>#4 2021 Carbon Edition Turbo · Ron Tonkin Honda</t>
+          <t>#14 2023 2.5 S Premium · Rodland Toyota</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -3577,93 +3485,56 @@
         </is>
       </c>
       <c r="F26" s="16" t="n">
-        <v>25852</v>
+        <v>28287</v>
       </c>
       <c r="G26" s="7" t="n"/>
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="16" t="n">
-        <v>29558.646</v>
+        <v>32028.848</v>
       </c>
       <c r="L26" s="16" t="n">
-        <v>575.5838348034372</v>
+        <v>623.6851023614681</v>
       </c>
       <c r="M26" s="16" t="n">
-        <v>478.2208103260242</v>
+        <v>526.3220778840551</v>
       </c>
       <c r="N26" s="16" t="n">
-        <v>4976.384088206229</v>
+        <v>5392.258141688082</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>#1 2023 2.5 Turbo AWD · Puyallup Mazda</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>est</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="n">
-        <v>27719</v>
-      </c>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="16" t="n">
-        <v>31512.652</v>
-      </c>
-      <c r="L27" s="16" t="n">
-        <v>613.6334216048396</v>
-      </c>
-      <c r="M27" s="16" t="n">
-        <v>516.2703971274266</v>
-      </c>
-      <c r="N27" s="16" t="n">
-        <v>5305.35329629037</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="25" t="inlineStr">
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="inlineStr">
         <is>
           <t>Δ</t>
         </is>
       </c>
-      <c r="D28" s="25" t="n"/>
-      <c r="E28" s="25" t="n"/>
-      <c r="F28" s="26" t="n">
-        <v>1867</v>
-      </c>
-      <c r="G28" s="25" t="n"/>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
-      <c r="J28" s="25" t="n"/>
-      <c r="K28" s="26" t="n">
-        <v>1954.006000000001</v>
-      </c>
-      <c r="L28" s="26" t="n">
-        <v>38.04958680140237</v>
-      </c>
-      <c r="M28" s="26" t="n">
-        <v>38.04958680140243</v>
-      </c>
-      <c r="N28" s="26" t="n">
-        <v>328.9692080841414</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="14" t="inlineStr">
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="26" t="n">
+        <v>2435</v>
+      </c>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
+      <c r="K27" s="26" t="n">
+        <v>2470.202000000001</v>
+      </c>
+      <c r="L27" s="26" t="n">
+        <v>48.10126755803094</v>
+      </c>
+      <c r="M27" s="26" t="n">
+        <v>48.101267558031</v>
+      </c>
+      <c r="N27" s="26" t="n">
+        <v>415.8740534818535</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Rule: cheapest solid = lowest estimated out-the-door figure among live cars with a verified 1-owner / 0-accident history (or Mazda CPO) at a franchise dealer; stretch = best-value live 2023 in the Turbo / Premium tiers, ranked by list price against KBB Seattle fair purchase price.</t>
         </is>
@@ -3681,7 +3552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O9"/>
+  <dimension ref="B1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" min="1" max="1"/>
@@ -3771,10 +3642,10 @@
     </row>
     <row r="4">
       <c r="B4" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
@@ -3783,63 +3654,63 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Acura of Seattle</t>
+          <t>Puyallup Mazda</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Tukwila, WA</t>
+          <t>Puyallup, WA</t>
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>27300</v>
+        <v>27919</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>25353</v>
+        <v>27990</v>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Aug 11</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>confirmed Aug 11 PM</t>
+          <t>purchased by the buyer this report was built for</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/451655500</t>
+          <t>https://www.cargurus.com/Cars/listing/448185375</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Grand Touring Reserve AWD (2.5 Turbo)</t>
+          <t>2.5 Turbo AWD</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>BMW Seattle</t>
+          <t>Acura of Seattle</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Tukwila, WA</t>
         </is>
       </c>
       <c r="G5" s="9" t="n">
-        <v>24999</v>
+        <v>27300</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>39141</v>
+        <v>25353</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -3848,130 +3719,130 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>dealer confirmed Aug 11 PM; CarGurus copy closed Aug 12</t>
+          <t>confirmed Aug 11 PM</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/455054228</t>
+          <t>https://www.cargurus.com/Cars/listing/451655500</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>2.5 S Preferred AWD</t>
+          <t>Grand Touring Reserve AWD (2.5 Turbo)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Royal Moore Mazda</t>
+          <t>BMW Seattle</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Hillsboro, OR</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>26900</v>
+        <v>24999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>16615</v>
+        <v>39141</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Aug 13</t>
+          <t>Aug 11</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>dealer email Aug 13</t>
+          <t>dealer confirmed Aug 11 PM; CarGurus copy closed Aug 12</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>https://www.cargurus.com/Cars/listing/454567468</t>
+          <t>https://www.cargurus.com/Cars/listing/455054228</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Carbon Edition</t>
+          <t>2.5 S Preferred AWD</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>CarMax Sacramento South</t>
+          <t>Royal Moore Mazda</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Hillsboro, OR</t>
         </is>
       </c>
       <c r="G7" s="9" t="n">
-        <v>24998</v>
+        <v>26900</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>48337</v>
+        <v>16615</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Aug 11</t>
+          <t>Aug 13</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Aug 11 PM</t>
+          <t>dealer email Aug 13</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>https://www.carmax.com/car/70056694</t>
+          <t>https://www.cargurus.com/Cars/listing/454567468</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Grand Touring AWD</t>
+          <t>Carbon Edition</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Doug's Lynnwood Mazda</t>
+          <t>CarMax Sacramento South</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Edmonds, WA</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>28700</v>
+        <v>24998</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>27089</v>
+        <v>48337</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
@@ -3980,54 +3851,98 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>dealer email Aug 11 (sold Aug 10)</t>
+          <t>Aug 11 PM</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>https://www.cars.com/vehicledetail/495a1e58-37a7-480b-9f80-8bb411d8fa8f/</t>
+          <t>https://www.carmax.com/car/70056694</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Grand Touring AWD</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Doug's Lynnwood Mazda</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Edmonds, WA</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>28700</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>27089</v>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Aug 11</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>dealer email Aug 11 (sold Aug 10)</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cars.com/vehicledetail/495a1e58-37a7-480b-9f80-8bb411d8fa8f/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C10" s="8" t="n">
         <v>2023</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>2.5 S Preferred AWD</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Auto Connections of Bellevue (independent)</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G10" s="9" t="n">
         <v>26495</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H10" s="6" t="n">
         <v>20533</v>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>Aug 11</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>Aug 11, 11:51 AM</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>https://www.cargurus.com/Cars/listing/450670232</t>
         </is>
@@ -5489,11 +5404,11 @@
         <v>30980</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>27919</v>
+        <v>28998</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>#1</t>
+          <t>CarGurus</t>
         </is>
       </c>
       <c r="H19" s="16">
@@ -5502,7 +5417,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">

</xml_diff>